<commit_message>
feat: update experiment data
</commit_message>
<xml_diff>
--- a/ExperimentsData.xlsx
+++ b/ExperimentsData.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamchristian/Documents/PersonalProjects/prethesis-experiments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\personal\prethesis-experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FFF86A7-9490-A04E-85A9-8D28DE90B825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF57B427-AD30-41D8-90F2-55BC75FD62FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
   </bookViews>
   <sheets>
-    <sheet name="January30th" sheetId="1" r:id="rId1"/>
-    <sheet name="February14th" sheetId="2" r:id="rId2"/>
-    <sheet name="February25th" sheetId="3" r:id="rId3"/>
+    <sheet name="Dataset Distribution" sheetId="4" r:id="rId1"/>
+    <sheet name="January30th" sheetId="1" r:id="rId2"/>
+    <sheet name="February14th" sheetId="2" r:id="rId3"/>
+    <sheet name="February25th" sheetId="3" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,6 +39,70 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>William Christian</author>
+  </authors>
+  <commentList>
+    <comment ref="B3" authorId="0" shapeId="0" xr:uid="{1955260D-C12B-4778-A126-397FD64E6E7B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>William Christian:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Dataset dair/ai-emotion merupakan sebuah dataset yang kami temukan dari website hugging face dimana ada 1825 lebih model di hugging face yang menggunakan dataset tersebut untuk melakukan training.
+Total data yang ada didalam dataset tersebut yaitu 16 ribu lebih dengan persebaran label untuk dataset masih tidak balance dengan data yang paling banyak untuk label happy/joy dan juga sad seperti dataset Twitter Data
+Dataset dapat diakses lebih dalam dari link ini: https://huggingface.co/datasets/dair-ai/emotionWilliam Christian:
+Dataset dair/ai-emotion merupakan sebuah dataset yang kami temukan dari website hugging face dimana ada 1825 lebih model di hugging face yang menggunakan dataset tersebut untuk melakukan training.
+Total data yang ada didalam dataset tersebut yaitu 16 ribu lebih dengan persebaran label untuk dataset masih tidak balance dengan data yang paling banyak untuk label happy/joy dan juga sad seperti dataset Twitter Data
+Dataset dapat diakses lebih dalam dari link ini: https://huggingface.co/datasets/dair-ai/emotion</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B15" authorId="0" shapeId="0" xr:uid="{AE80D999-32DC-406E-8A0D-944FE9E6C4F5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>William Christian:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Dataset Twitter mempunyai total 9870 data, yang mempunyai persebaran lable yang tidak balance (dengan data yang sangat banyak untuk dataset dengan label happy dan juga sad). Sehingga Augmentasi lebih memfokuskan penambahan data untuk label yang lain.
+Dataset diatas diakses dari link: https://www.kaggle.com/code/shainy/twitter-emotion-analysis/input</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Microsoft Office User</author>
@@ -82,7 +147,7 @@
 </comments>
 </file>
 
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>William Christian</author>
@@ -252,7 +317,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="34">
   <si>
     <t>DistilBERT</t>
   </si>
@@ -321,13 +386,46 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Label</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>sadness</t>
+  </si>
+  <si>
+    <t>anger</t>
+  </si>
+  <si>
+    <t>love</t>
+  </si>
+  <si>
+    <t>surprise</t>
+  </si>
+  <si>
+    <t>feat</t>
+  </si>
+  <si>
+    <t>joy</t>
+  </si>
+  <si>
+    <t>Twitter Data</t>
+  </si>
+  <si>
+    <t>disgust</t>
+  </si>
+  <si>
+    <t>fear</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -399,8 +497,29 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -425,8 +544,14 @@
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -467,19 +592,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -497,12 +632,6 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -510,11 +639,57 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="38">
+  <dxfs count="39">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
     <dxf>
       <border outline="0">
         <left style="thin">
@@ -1119,70 +1294,92 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}" name="Table1" displayName="Table1" ref="B3:H8" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
-  <autoFilter ref="B3:H8" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{4978B2AE-4B4B-EA49-BF70-5AABACA85971}" name="Dataset Name" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{58D50865-DFF7-8644-AD30-63D47540D02C}" name="Accuracy" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{BBA594A0-A636-D445-AAB9-22C6754D09C0}" name="Precision" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{661E434A-CCB1-BB46-BA1D-8A2D641D7D25}" name="Recall" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{A58BD05A-F5EB-AF4E-A041-498A7ACF41DE}" name="F1" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{B40DA81D-2CB3-F14B-8186-F7D0A18BA0FE}" name="Loss" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{83055B2D-4E00-F845-BC1B-6F22C502B5D2}" name="Epoch" dataDxfId="29"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{306760BC-4A86-48F5-9CF5-A85404614954}" name="Table8" displayName="Table8" ref="B4:C10" totalsRowShown="0">
+  <autoFilter ref="B4:C10" xr:uid="{306760BC-4A86-48F5-9CF5-A85404614954}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{C071879A-DF9F-4E65-8142-32166A9804FE}" name="Label"/>
+    <tableColumn id="2" xr3:uid="{2BB1A1D5-B219-42D6-B570-666165AC385E}" name="Amount"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}" name="Table13" displayName="Table13" ref="J12:P18" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
-  <autoFilter ref="J12:P18" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{EAE6D8E7-8EF0-D94F-A26B-7A025E6C7361}" name="Dataset Name" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{36A28C87-4153-404C-A82A-6C01A5B3DC55}" name="Accuracy" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{E4A45E88-BACC-B941-A1C0-4BBCB2A3CAB7}" name="Precision" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{0106A244-4E6C-994C-8E0B-A39D4088698B}" name="Recall" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{B4A28C88-CF22-604F-982B-A6A1CCF1A1F7}" name="F1" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{0CBF8E57-666D-A545-BA88-90DE39497A4E}" name="Loss" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{944AF69F-9D99-0548-9A49-04236D354F4E}" name="Epoch" dataDxfId="20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{33D6D3E5-9AAF-4914-BE32-298E922BC8A4}" name="Table9" displayName="Table9" ref="B16:C22" totalsRowShown="0">
+  <autoFilter ref="B16:C22" xr:uid="{33D6D3E5-9AAF-4914-BE32-298E922BC8A4}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{5155CECE-BBA4-45F8-98E3-DD9D18244FF8}" name="Label" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{6A1175E6-E870-42B6-8AC2-1516761E3F86}" name="Amount"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}" name="Table134" displayName="Table134" ref="B11:H16" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
-  <autoFilter ref="B11:H16" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}" name="Table1" displayName="Table1" ref="B3:H8" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
+  <autoFilter ref="B3:H8" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{05A1D84A-55CA-EA40-A483-5E78D383B19B}" name="Dataset Name" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{CA820C5C-5B52-894C-A49F-0549BA14EB14}" name="Accuracy" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{23F3C118-B36A-8344-91C4-91E68C152060}" name="Precision" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{3FDE3D07-7EC9-814A-B04A-1749B565F6EA}" name="Recall" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{4E62075D-7975-3747-9112-6DA05E872576}" name="F1" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{E6B084A9-1443-8E43-8957-DF1E2A9B10B8}" name="Loss" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{AB463B29-B751-9A41-A7DB-1E69264E687D}" name="Epoch" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{4978B2AE-4B4B-EA49-BF70-5AABACA85971}" name="Dataset Name" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{58D50865-DFF7-8644-AD30-63D47540D02C}" name="Accuracy" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{BBA594A0-A636-D445-AAB9-22C6754D09C0}" name="Precision" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{661E434A-CCB1-BB46-BA1D-8A2D641D7D25}" name="Recall" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{A58BD05A-F5EB-AF4E-A041-498A7ACF41DE}" name="F1" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{B40DA81D-2CB3-F14B-8186-F7D0A18BA0FE}" name="Loss" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{83055B2D-4E00-F845-BC1B-6F22C502B5D2}" name="Epoch" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}" name="Table7" displayName="Table7" ref="J3:P5" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
-  <autoFilter ref="J3:P5" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}" name="Table13" displayName="Table13" ref="J12:P18" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+  <autoFilter ref="J12:P18" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{F2E57A4A-2AAD-7447-91C9-007605371819}" name="Model" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{CB02CB06-53A1-2F41-AD51-1547D4DC27A1}" name="Accuracy" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{CA4460C1-43B3-7449-A208-84080D817025}" name="Precision" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{1367CE74-9216-4149-A489-1B4EB4644578}" name="Recall" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{9CF0E2A6-FC0C-744D-AC36-893DD9641356}" name="F1" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{913D2EB3-6EB7-6D45-9EE3-E045E761BD2B}" name="Loss" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{8C15DD0C-3E42-5C44-92F8-BD590893AE2E}" name="Epoch" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{EAE6D8E7-8EF0-D94F-A26B-7A025E6C7361}" name="Dataset Name" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{36A28C87-4153-404C-A82A-6C01A5B3DC55}" name="Accuracy" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{E4A45E88-BACC-B941-A1C0-4BBCB2A3CAB7}" name="Precision" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{0106A244-4E6C-994C-8E0B-A39D4088698B}" name="Recall" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{B4A28C88-CF22-604F-982B-A6A1CCF1A1F7}" name="F1" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{0CBF8E57-666D-A545-BA88-90DE39497A4E}" name="Loss" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{944AF69F-9D99-0548-9A49-04236D354F4E}" name="Epoch" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}" name="Table134" displayName="Table134" ref="B11:H16" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+  <autoFilter ref="B11:H16" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{05A1D84A-55CA-EA40-A483-5E78D383B19B}" name="Dataset Name" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{CA820C5C-5B52-894C-A49F-0549BA14EB14}" name="Accuracy" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{23F3C118-B36A-8344-91C4-91E68C152060}" name="Precision" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{3FDE3D07-7EC9-814A-B04A-1749B565F6EA}" name="Recall" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{4E62075D-7975-3747-9112-6DA05E872576}" name="F1" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{E6B084A9-1443-8E43-8957-DF1E2A9B10B8}" name="Loss" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{AB463B29-B751-9A41-A7DB-1E69264E687D}" name="Epoch" dataDxfId="12"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}" name="Table7" displayName="Table7" ref="J3:P5" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="J3:P5" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{F2E57A4A-2AAD-7447-91C9-007605371819}" name="Model" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{CB02CB06-53A1-2F41-AD51-1547D4DC27A1}" name="Accuracy" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{CA4460C1-43B3-7449-A208-84080D817025}" name="Precision" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{1367CE74-9216-4149-A489-1B4EB4644578}" name="Recall" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{9CF0E2A6-FC0C-744D-AC36-893DD9641356}" name="F1" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{913D2EB3-6EB7-6D45-9EE3-E045E761BD2B}" name="Loss" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{8C15DD0C-3E42-5C44-92F8-BD590893AE2E}" name="Epoch" dataDxfId="3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{72514C95-6960-EE4E-9C9E-993ED7B9BAC1}" name="Table16" displayName="Table16" ref="B3:H6" totalsRowShown="0">
   <autoFilter ref="B3:H6" xr:uid="{72514C95-6960-EE4E-9C9E-993ED7B9BAC1}"/>
   <tableColumns count="7">
@@ -1198,7 +1395,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{DDD656AE-FBAE-6646-B9F6-53768524C098}" name="Table137" displayName="Table137" ref="B10:H15" totalsRowShown="0">
   <autoFilter ref="B10:H15" xr:uid="{DDD656AE-FBAE-6646-B9F6-53768524C098}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B11:H15">
@@ -1217,8 +1414,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{372BED72-405E-1348-A031-F1B0B5AE3EF5}" name="Table4" displayName="Table4" ref="B19:I23" totalsRowShown="0" headerRowDxfId="1" tableBorderDxfId="0">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{372BED72-405E-1348-A031-F1B0B5AE3EF5}" name="Table4" displayName="Table4" ref="B19:I23" totalsRowShown="0" headerRowDxfId="2" tableBorderDxfId="1">
   <autoFilter ref="B19:I23" xr:uid="{372BED72-405E-1348-A031-F1B0B5AE3EF5}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{1A099EFA-B86F-3A4E-BCA0-D958972A588E}" name="Model"/>
@@ -1550,32 +1747,179 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F41AEED8-ECB9-41F9-BCFE-8D94D2C04651}">
+  <dimension ref="B3:C22"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="20"/>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5">
+        <v>5797</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6">
+        <v>2709</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7">
+        <v>1641</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9">
+        <v>2373</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10">
+        <v>6761</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B15" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="20"/>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17">
+        <v>2849</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="19" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B22" s="18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22">
+        <v>3928</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B15:C15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14964B3B-3353-C742-BCAB-B2A6487822EC}">
   <dimension ref="B2:P19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="2"/>
-    <col min="2" max="2" width="28.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.125" style="2"/>
+    <col min="2" max="2" width="28.375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.375" style="2" customWidth="1"/>
     <col min="4" max="4" width="10.5" style="2" customWidth="1"/>
-    <col min="5" max="9" width="9.1640625" style="2"/>
-    <col min="10" max="10" width="24.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="9" width="9.125" style="2"/>
+    <col min="10" max="10" width="24.875" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11" style="2" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="10.875" style="2" customWidth="1"/>
     <col min="13" max="15" width="10.5" style="2" customWidth="1"/>
-    <col min="16" max="16384" width="9.1640625" style="2"/>
+    <col min="16" max="16384" width="9.125" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B2" s="1" t="s">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B2" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="J2" s="3" t="s">
+      <c r="C2" s="15"/>
+      <c r="J2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1619,7 +1963,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
@@ -1644,145 +1988,145 @@
       <c r="J4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="3">
         <v>0.63333333333333297</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="3">
         <v>0.58940855146517701</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="3">
         <v>0.57971965210112997</v>
       </c>
-      <c r="N4" s="4">
+      <c r="N4" s="3">
         <v>0.58123915300385798</v>
       </c>
-      <c r="O4" s="4">
+      <c r="O4" s="3">
         <v>1.98164403438568</v>
       </c>
       <c r="P4" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B5" s="5" t="s">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>0.94199999999999995</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>0.91009287368524705</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <v>0.92115560716326905</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="4">
         <v>0.91533564022587399</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="4">
         <v>0.191635861992836</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="4">
         <v>3</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="3">
         <v>0.65370370370370301</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="3">
         <v>0.61064478919585496</v>
       </c>
-      <c r="M5" s="4">
+      <c r="M5" s="3">
         <v>0.61110922657225697</v>
       </c>
-      <c r="N5" s="4">
+      <c r="N5" s="3">
         <v>0.60562519999897302</v>
       </c>
-      <c r="O5" s="4">
+      <c r="O5" s="3">
         <v>2.0909550189971902</v>
       </c>
       <c r="P5" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="2">
         <v>0.90110000000000001</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>0.88689723831664402</v>
       </c>
       <c r="E6" s="2">
         <v>0.89348445507910701</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="3">
         <v>0.88892574969448901</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="3">
         <v>0.46213433146476701</v>
       </c>
       <c r="H6" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="5">
         <v>0.9355</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="5">
         <v>0.90203298486156802</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="5">
         <v>0.90715039969428501</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="5">
         <v>0.90403925299948695</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="5">
         <v>0.47319608926772999</v>
       </c>
       <c r="H7" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <v>0.94799999999999995</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="5">
         <v>0.94802861178020803</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="5">
         <v>0.94798241355127499</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="5">
         <v>0.94790593102700604</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="5">
         <v>0.37256675958633401</v>
       </c>
       <c r="H8" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B10" s="3" t="s">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="3"/>
-    </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="C10" s="1"/>
+    </row>
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>2</v>
       </c>
@@ -1804,28 +2148,28 @@
       <c r="H11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="J11" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K11" s="3"/>
-    </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="K11" s="1"/>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="3">
         <v>0.96199999999999997</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12" s="3">
         <v>0.96304908720007598</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12" s="3">
         <v>0.96197694700688696</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12" s="3">
         <v>0.96186219945891205</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="3">
         <v>0.139405786991119</v>
       </c>
       <c r="H12" s="2">
@@ -1853,96 +2197,96 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B13" s="5" t="s">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="6">
         <v>0.94299999999999995</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="6">
         <v>0.917014698774683</v>
       </c>
-      <c r="E13" s="7">
+      <c r="E13" s="6">
         <v>0.91827723390579796</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F13" s="6">
         <v>0.917529975022639</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="6">
         <v>0.18735474348068201</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="4">
         <v>3</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="K13" s="4">
+      <c r="K13" s="3">
         <v>0.95899999999999996</v>
       </c>
-      <c r="L13" s="4">
+      <c r="L13" s="3">
         <v>0.95988468893644996</v>
       </c>
-      <c r="M13" s="4">
+      <c r="M13" s="3">
         <v>0.95898143652634604</v>
       </c>
-      <c r="N13" s="4">
+      <c r="N13" s="3">
         <v>0.95889844821641901</v>
       </c>
-      <c r="O13" s="4">
+      <c r="O13" s="3">
         <v>0.16755579411983401</v>
       </c>
       <c r="P13" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C14" s="3">
         <v>0.91017964071856206</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <v>0.90220869383463398</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="3">
         <v>0.89460743976516799</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F14" s="3">
         <v>0.89720299182954899</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14" s="3">
         <v>0.38670238852500899</v>
       </c>
       <c r="H14" s="2">
         <v>3</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="6">
         <v>0.93700000000000006</v>
       </c>
-      <c r="L14" s="7">
+      <c r="L14" s="6">
         <v>0.92557082683330705</v>
       </c>
-      <c r="M14" s="7">
+      <c r="M14" s="6">
         <v>0.90349649643238195</v>
       </c>
-      <c r="N14" s="7">
+      <c r="N14" s="6">
         <v>0.91098762484752904</v>
       </c>
-      <c r="O14" s="7">
+      <c r="O14" s="6">
         <v>0.17923152446746801</v>
       </c>
-      <c r="P14" s="5">
+      <c r="P14" s="4">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B15" s="5" t="s">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B15" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="2">
@@ -1966,26 +2310,26 @@
       <c r="J15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K15" s="4">
+      <c r="K15" s="3">
         <v>0.89720558882235502</v>
       </c>
-      <c r="L15" s="4">
+      <c r="L15" s="3">
         <v>0.91434566130830597</v>
       </c>
-      <c r="M15" s="4">
+      <c r="M15" s="3">
         <v>0.88788730618628497</v>
       </c>
-      <c r="N15" s="4">
+      <c r="N15" s="3">
         <v>0.89892356840659804</v>
       </c>
-      <c r="O15" s="4">
+      <c r="O15" s="3">
         <v>0.46178486943244901</v>
       </c>
       <c r="P15" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>10</v>
       </c>
@@ -2014,7 +2358,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="J17" s="2" t="s">
         <v>10</v>
       </c>
@@ -2037,7 +2381,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:C2"/>
@@ -2053,26 +2397,26 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{480C1162-B378-5D47-92C7-5997231863D1}">
   <dimension ref="B2:I23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.375" customWidth="1"/>
     <col min="5" max="5" width="10.5" customWidth="1"/>
     <col min="9" max="9" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B2" s="8" t="s">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>9</v>
       </c>
@@ -2095,7 +2439,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>11</v>
       </c>
@@ -2118,7 +2462,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>0</v>
       </c>
@@ -2141,7 +2485,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -2164,12 +2508,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B9" s="9" t="s">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>9</v>
       </c>
@@ -2192,7 +2536,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>0</v>
       </c>
@@ -2215,7 +2559,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>0</v>
       </c>
@@ -2238,7 +2582,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>11</v>
       </c>
@@ -2261,7 +2605,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>16</v>
       </c>
@@ -2284,7 +2628,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>16</v>
       </c>
@@ -2307,91 +2651,91 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B18" s="10" t="s">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="10"/>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="11" t="s">
+      <c r="C18" s="17"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C19" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="11" t="s">
+      <c r="D19" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H19" s="12" t="s">
+      <c r="H19" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="I19" s="13" t="s">
+      <c r="I19" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B20" s="14" t="s">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="11">
         <v>1.26833808422088</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="11">
         <v>0.67777777777777704</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="11">
         <v>0.63890078720888599</v>
       </c>
-      <c r="F20" s="14">
+      <c r="F20" s="11">
         <v>0.63380646955689901</v>
       </c>
-      <c r="G20" s="14">
+      <c r="G20" s="11">
         <v>0.63609223650959501</v>
       </c>
-      <c r="H20" s="15">
+      <c r="H20" s="12">
         <v>4</v>
       </c>
       <c r="I20" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B21" s="16" t="s">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C21" s="16">
+      <c r="C21" s="13">
         <v>1.5849186182021999</v>
       </c>
-      <c r="D21" s="16">
+      <c r="D21" s="13">
         <v>0.66857142857142804</v>
       </c>
-      <c r="E21" s="16">
+      <c r="E21" s="13">
         <v>0.672903537266902</v>
       </c>
-      <c r="F21" s="16">
+      <c r="F21" s="13">
         <v>0.66857142857142804</v>
       </c>
-      <c r="G21" s="16">
+      <c r="G21" s="13">
         <v>0.67013161896733497</v>
       </c>
-      <c r="H21" s="17">
+      <c r="H21" s="14">
         <v>4</v>
       </c>
       <c r="I21" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>13</v>
       </c>
@@ -2417,7 +2761,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>13</v>
       </c>
@@ -2458,10 +2802,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F95E52D2-75E8-D44D-9380-8EC3BF1C86A2}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: update experiments data
</commit_message>
<xml_diff>
--- a/ExperimentsData.xlsx
+++ b/ExperimentsData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\personal\prethesis-experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF57B427-AD30-41D8-90F2-55BC75FD62FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F8A35CE-1806-4A72-B73B-E133120736EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="3" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Distribution" sheetId="4" r:id="rId1"/>
@@ -317,7 +317,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="37">
   <si>
     <t>DistilBERT</t>
   </si>
@@ -420,6 +420,15 @@
   <si>
     <t>fear</t>
   </si>
+  <si>
+    <t>Models</t>
+  </si>
+  <si>
+    <t>Twitter Dataset</t>
+  </si>
+  <si>
+    <t>Indonesian Dataset</t>
+  </si>
 </sst>
 </file>
 
@@ -519,7 +528,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -550,8 +559,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -605,11 +620,117 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -639,6 +760,23 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -648,9 +786,16 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -658,38 +803,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="39">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
     <dxf>
       <border outline="0">
         <left style="thin">
@@ -1280,6 +1393,38 @@
       </font>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1293,6 +1438,461 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>800100</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>809625</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>159544</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9DA23D64-7161-5880-A3FD-0AE896AD163F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1638300" y="1628775"/>
+          <a:ext cx="4200525" cy="3150394"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0773276A-D7BA-1312-C9F4-653A28CC49F0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1714500" y="5229225"/>
+          <a:ext cx="4152900" cy="3114675"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>157163</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7A4A72B9-E817-2DFC-0238-FB717BAE2A6B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1676400" y="8820150"/>
+          <a:ext cx="4210050" cy="3157538"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>819150</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>128588</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8CF8E60F-F6C8-6978-FDF8-84671A7094D7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9220200" y="1619250"/>
+          <a:ext cx="4171950" cy="3128963"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6FE3C25B-3ACB-B2E4-328E-9808C06F66CA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9220200" y="5219700"/>
+          <a:ext cx="4191000" cy="3143250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A05CC5BD-68FF-524A-333E-0BFE120AF35A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9220200" y="8820150"/>
+          <a:ext cx="4114800" cy="3086100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>447675</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>64294</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 14">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11112CB6-8689-703C-901F-A07452F6873A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16373475" y="1657350"/>
+          <a:ext cx="4314825" cy="3236119"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Picture 16">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B0DC632-1CD9-92FB-9DB9-E1A35F314C29}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16440150" y="5391150"/>
+          <a:ext cx="4152900" cy="3114675"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>647700</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Picture 18">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A7BCFB2-05E3-0154-294D-308A0F408429}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="16573500" y="8991600"/>
+          <a:ext cx="4076700" cy="3057525"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{306760BC-4A86-48F5-9CF5-A85404614954}" name="Table8" displayName="Table8" ref="B4:C10" totalsRowShown="0">
   <autoFilter ref="B4:C10" xr:uid="{306760BC-4A86-48F5-9CF5-A85404614954}"/>
@@ -1304,11 +1904,58 @@
 </table>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F6EB79E9-0B6F-42C2-8611-8D0E6CF90686}" name="Table10" displayName="Table10" ref="B3:H6" totalsRowShown="0">
+  <autoFilter ref="B3:H6" xr:uid="{F6EB79E9-0B6F-42C2-8611-8D0E6CF90686}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{E0D099F3-710D-42CC-BCA1-4C3C1AE43E43}" name="Models"/>
+    <tableColumn id="2" xr3:uid="{2AB1B627-41DE-4113-92F7-574CC093B57C}" name="Loss"/>
+    <tableColumn id="3" xr3:uid="{81C6AC62-F1F8-4F5F-80DF-2632C4A3CBC4}" name="Accuracy"/>
+    <tableColumn id="4" xr3:uid="{A8553EA8-8D26-40B4-A356-84BF46974F44}" name="Precision"/>
+    <tableColumn id="5" xr3:uid="{40D86159-4A75-4EBF-B172-01D7BCC33969}" name="Recall"/>
+    <tableColumn id="6" xr3:uid="{BA3C992D-D9A0-42A6-86F7-0429FE50A20F}" name="F1"/>
+    <tableColumn id="7" xr3:uid="{E4260AC9-9A76-4F02-9F84-709C693D749B}" name="Epoch"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{D312D647-6FD7-4879-8EE5-33E0DC375794}" name="Table1012" displayName="Table1012" ref="K3:Q6" totalsRowShown="0">
+  <autoFilter ref="K3:Q6" xr:uid="{D312D647-6FD7-4879-8EE5-33E0DC375794}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{0BC9DE4D-62EA-46F6-8431-066E446B4A73}" name="Models"/>
+    <tableColumn id="2" xr3:uid="{6007322B-CD34-49AD-921C-C13680A6A881}" name="Loss"/>
+    <tableColumn id="3" xr3:uid="{94EC1D78-F934-4793-B66D-E289F915D70E}" name="Accuracy"/>
+    <tableColumn id="4" xr3:uid="{407C858F-C1CE-4801-9502-27C879C87376}" name="Precision"/>
+    <tableColumn id="5" xr3:uid="{32ACFDEE-A7B8-4302-9100-78907542F005}" name="Recall"/>
+    <tableColumn id="6" xr3:uid="{B5A53498-CBB5-486C-A71E-D77AD1B1F4DD}" name="F1"/>
+    <tableColumn id="7" xr3:uid="{063654CC-B77D-4A7C-ABE3-003CF0DD5016}" name="Epoch"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{7FBE2E18-5676-435C-908A-B567841F99FA}" name="Table12" displayName="Table12" ref="T3:Y6" totalsRowShown="0">
+  <autoFilter ref="T3:Y6" xr:uid="{7FBE2E18-5676-435C-908A-B567841F99FA}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{C9CFB6E4-FCE0-452B-9965-D56F453B1B99}" name="Epoch"/>
+    <tableColumn id="2" xr3:uid="{4F290C5F-074D-4CAA-82F1-07C356451070}" name="Loss"/>
+    <tableColumn id="3" xr3:uid="{88475986-A652-4EBC-8FF2-7E38AA14540D}" name="Accuracy"/>
+    <tableColumn id="4" xr3:uid="{14F22B62-0C7D-4B65-8BA8-9B2938E61906}" name="Precision"/>
+    <tableColumn id="5" xr3:uid="{6E9009F6-2DFF-4C42-A561-F3FBBD7F3428}" name="Recall"/>
+    <tableColumn id="6" xr3:uid="{5B4A95EF-D5E0-4EAD-8C1B-39D5378D5C4F}" name="F1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{33D6D3E5-9AAF-4914-BE32-298E922BC8A4}" name="Table9" displayName="Table9" ref="B16:C22" totalsRowShown="0">
   <autoFilter ref="B16:C22" xr:uid="{33D6D3E5-9AAF-4914-BE32-298E922BC8A4}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{5155CECE-BBA4-45F8-98E3-DD9D18244FF8}" name="Label" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{5155CECE-BBA4-45F8-98E3-DD9D18244FF8}" name="Label" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{6A1175E6-E870-42B6-8AC2-1516761E3F86}" name="Amount"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1316,64 +1963,64 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}" name="Table1" displayName="Table1" ref="B3:H8" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}" name="Table1" displayName="Table1" ref="B3:H8" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
   <autoFilter ref="B3:H8" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{4978B2AE-4B4B-EA49-BF70-5AABACA85971}" name="Dataset Name" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{58D50865-DFF7-8644-AD30-63D47540D02C}" name="Accuracy" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{BBA594A0-A636-D445-AAB9-22C6754D09C0}" name="Precision" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{661E434A-CCB1-BB46-BA1D-8A2D641D7D25}" name="Recall" dataDxfId="33"/>
-    <tableColumn id="5" xr3:uid="{A58BD05A-F5EB-AF4E-A041-498A7ACF41DE}" name="F1" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{B40DA81D-2CB3-F14B-8186-F7D0A18BA0FE}" name="Loss" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{83055B2D-4E00-F845-BC1B-6F22C502B5D2}" name="Epoch" dataDxfId="30"/>
+    <tableColumn id="1" xr3:uid="{4978B2AE-4B4B-EA49-BF70-5AABACA85971}" name="Dataset Name" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{58D50865-DFF7-8644-AD30-63D47540D02C}" name="Accuracy" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{BBA594A0-A636-D445-AAB9-22C6754D09C0}" name="Precision" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{661E434A-CCB1-BB46-BA1D-8A2D641D7D25}" name="Recall" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{A58BD05A-F5EB-AF4E-A041-498A7ACF41DE}" name="F1" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{B40DA81D-2CB3-F14B-8186-F7D0A18BA0FE}" name="Loss" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{83055B2D-4E00-F845-BC1B-6F22C502B5D2}" name="Epoch" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}" name="Table13" displayName="Table13" ref="J12:P18" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}" name="Table13" displayName="Table13" ref="J12:P18" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
   <autoFilter ref="J12:P18" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{EAE6D8E7-8EF0-D94F-A26B-7A025E6C7361}" name="Dataset Name" dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{36A28C87-4153-404C-A82A-6C01A5B3DC55}" name="Accuracy" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{E4A45E88-BACC-B941-A1C0-4BBCB2A3CAB7}" name="Precision" dataDxfId="25"/>
-    <tableColumn id="4" xr3:uid="{0106A244-4E6C-994C-8E0B-A39D4088698B}" name="Recall" dataDxfId="24"/>
-    <tableColumn id="5" xr3:uid="{B4A28C88-CF22-604F-982B-A6A1CCF1A1F7}" name="F1" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{0CBF8E57-666D-A545-BA88-90DE39497A4E}" name="Loss" dataDxfId="22"/>
-    <tableColumn id="7" xr3:uid="{944AF69F-9D99-0548-9A49-04236D354F4E}" name="Epoch" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{EAE6D8E7-8EF0-D94F-A26B-7A025E6C7361}" name="Dataset Name" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{36A28C87-4153-404C-A82A-6C01A5B3DC55}" name="Accuracy" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{E4A45E88-BACC-B941-A1C0-4BBCB2A3CAB7}" name="Precision" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{0106A244-4E6C-994C-8E0B-A39D4088698B}" name="Recall" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{B4A28C88-CF22-604F-982B-A6A1CCF1A1F7}" name="F1" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{0CBF8E57-666D-A545-BA88-90DE39497A4E}" name="Loss" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{944AF69F-9D99-0548-9A49-04236D354F4E}" name="Epoch" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}" name="Table134" displayName="Table134" ref="B11:H16" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}" name="Table134" displayName="Table134" ref="B11:H16" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="B11:H16" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{05A1D84A-55CA-EA40-A483-5E78D383B19B}" name="Dataset Name" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{CA820C5C-5B52-894C-A49F-0549BA14EB14}" name="Accuracy" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{23F3C118-B36A-8344-91C4-91E68C152060}" name="Precision" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{3FDE3D07-7EC9-814A-B04A-1749B565F6EA}" name="Recall" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{4E62075D-7975-3747-9112-6DA05E872576}" name="F1" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{E6B084A9-1443-8E43-8957-DF1E2A9B10B8}" name="Loss" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{AB463B29-B751-9A41-A7DB-1E69264E687D}" name="Epoch" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{05A1D84A-55CA-EA40-A483-5E78D383B19B}" name="Dataset Name" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{CA820C5C-5B52-894C-A49F-0549BA14EB14}" name="Accuracy" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{23F3C118-B36A-8344-91C4-91E68C152060}" name="Precision" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{3FDE3D07-7EC9-814A-B04A-1749B565F6EA}" name="Recall" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{4E62075D-7975-3747-9112-6DA05E872576}" name="F1" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{E6B084A9-1443-8E43-8957-DF1E2A9B10B8}" name="Loss" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{AB463B29-B751-9A41-A7DB-1E69264E687D}" name="Epoch" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}" name="Table7" displayName="Table7" ref="J3:P5" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}" name="Table7" displayName="Table7" ref="J3:P5" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="J3:P5" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{F2E57A4A-2AAD-7447-91C9-007605371819}" name="Model" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{CB02CB06-53A1-2F41-AD51-1547D4DC27A1}" name="Accuracy" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{CA4460C1-43B3-7449-A208-84080D817025}" name="Precision" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{1367CE74-9216-4149-A489-1B4EB4644578}" name="Recall" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{9CF0E2A6-FC0C-744D-AC36-893DD9641356}" name="F1" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{913D2EB3-6EB7-6D45-9EE3-E045E761BD2B}" name="Loss" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{8C15DD0C-3E42-5C44-92F8-BD590893AE2E}" name="Epoch" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{F2E57A4A-2AAD-7447-91C9-007605371819}" name="Model" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{CB02CB06-53A1-2F41-AD51-1547D4DC27A1}" name="Accuracy" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{CA4460C1-43B3-7449-A208-84080D817025}" name="Precision" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{1367CE74-9216-4149-A489-1B4EB4644578}" name="Recall" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{9CF0E2A6-FC0C-744D-AC36-893DD9641356}" name="F1" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{913D2EB3-6EB7-6D45-9EE3-E045E761BD2B}" name="Loss" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{8C15DD0C-3E42-5C44-92F8-BD590893AE2E}" name="Epoch" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1415,7 +2062,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{372BED72-405E-1348-A031-F1B0B5AE3EF5}" name="Table4" displayName="Table4" ref="B19:I23" totalsRowShown="0" headerRowDxfId="2" tableBorderDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{372BED72-405E-1348-A031-F1B0B5AE3EF5}" name="Table4" displayName="Table4" ref="B19:I23" totalsRowShown="0" headerRowDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="B19:I23" xr:uid="{372BED72-405E-1348-A031-F1B0B5AE3EF5}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{1A099EFA-B86F-3A4E-BCA0-D958972A588E}" name="Model"/>
@@ -1756,10 +2403,10 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="20"/>
+      <c r="C3" s="29"/>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
@@ -1818,10 +2465,10 @@
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B15" s="20" t="s">
+      <c r="B15" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="20"/>
+      <c r="C15" s="29"/>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
@@ -1832,7 +2479,7 @@
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="16" t="s">
         <v>25</v>
       </c>
       <c r="C17">
@@ -1840,7 +2487,7 @@
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="15" t="s">
         <v>26</v>
       </c>
       <c r="C18">
@@ -1848,7 +2495,7 @@
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="16" t="s">
         <v>32</v>
       </c>
       <c r="C19">
@@ -1856,7 +2503,7 @@
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="15" t="s">
         <v>28</v>
       </c>
       <c r="C20">
@@ -1864,7 +2511,7 @@
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="16" t="s">
         <v>33</v>
       </c>
       <c r="C21">
@@ -1872,7 +2519,7 @@
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="15" t="s">
         <v>30</v>
       </c>
       <c r="C22">
@@ -1911,10 +2558,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="15"/>
+      <c r="C2" s="30"/>
       <c r="J2" s="1" t="s">
         <v>1</v>
       </c>
@@ -2410,11 +3057,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
@@ -2652,10 +3299,10 @@
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="17"/>
+      <c r="C18" s="32"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
@@ -2804,9 +3451,772 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F95E52D2-75E8-D44D-9380-8EC3BF1C86A2}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:Y62"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="34"/>
+      <c r="K2" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" s="34"/>
+      <c r="T2" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="U2" s="36"/>
+    </row>
+    <row r="3" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" t="s">
+        <v>8</v>
+      </c>
+      <c r="K3" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" t="s">
+        <v>7</v>
+      </c>
+      <c r="M3" t="s">
+        <v>3</v>
+      </c>
+      <c r="N3" t="s">
+        <v>4</v>
+      </c>
+      <c r="O3" t="s">
+        <v>5</v>
+      </c>
+      <c r="P3" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>8</v>
+      </c>
+      <c r="T3" t="s">
+        <v>8</v>
+      </c>
+      <c r="U3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V3" t="s">
+        <v>3</v>
+      </c>
+      <c r="W3" t="s">
+        <v>4</v>
+      </c>
+      <c r="X3" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <v>0.14634193480014801</v>
+      </c>
+      <c r="D4">
+        <v>0.97634011090573003</v>
+      </c>
+      <c r="E4">
+        <v>0.97636300426269895</v>
+      </c>
+      <c r="F4">
+        <v>0.97633463854631897</v>
+      </c>
+      <c r="G4">
+        <v>0.97633463854631897</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+      <c r="K4" t="s">
+        <v>11</v>
+      </c>
+      <c r="L4">
+        <v>0.30560222268104498</v>
+      </c>
+      <c r="M4">
+        <v>0.94720101781170396</v>
+      </c>
+      <c r="N4">
+        <v>0.94796661307067998</v>
+      </c>
+      <c r="O4">
+        <v>0.94720101781170496</v>
+      </c>
+      <c r="P4">
+        <v>0.94742140062100999</v>
+      </c>
+      <c r="Q4">
+        <v>4</v>
+      </c>
+      <c r="T4">
+        <v>4</v>
+      </c>
+      <c r="U4">
+        <v>1.14815354347229</v>
+      </c>
+      <c r="V4">
+        <v>0.77514124293785303</v>
+      </c>
+      <c r="W4">
+        <v>0.77738411519736295</v>
+      </c>
+      <c r="X4">
+        <v>0.77514124293785303</v>
+      </c>
+      <c r="Y4">
+        <v>0.77562753371646298</v>
+      </c>
+    </row>
+    <row r="5" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0.14440409839153201</v>
+      </c>
+      <c r="D5">
+        <v>0.97744916820702399</v>
+      </c>
+      <c r="E5">
+        <v>0.97744244340745801</v>
+      </c>
+      <c r="F5">
+        <v>0.97744574480172697</v>
+      </c>
+      <c r="G5">
+        <v>0.97743902804341998</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="K5" t="s">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0.31567558646201999</v>
+      </c>
+      <c r="M5">
+        <v>0.94656488549618301</v>
+      </c>
+      <c r="N5">
+        <v>0.94714816552521097</v>
+      </c>
+      <c r="O5">
+        <v>0.94656488549618301</v>
+      </c>
+      <c r="P5">
+        <v>0.94664828451880501</v>
+      </c>
+      <c r="Q5">
+        <v>4</v>
+      </c>
+      <c r="T5">
+        <v>10</v>
+      </c>
+      <c r="U5">
+        <v>1.6304794549942001</v>
+      </c>
+      <c r="V5">
+        <v>0.78757062146892598</v>
+      </c>
+      <c r="W5">
+        <v>0.78854656689159897</v>
+      </c>
+      <c r="X5">
+        <v>0.78757062146892598</v>
+      </c>
+      <c r="Y5">
+        <v>0.78763665437576802</v>
+      </c>
+    </row>
+    <row r="6" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6">
+        <v>0.14479537308216001</v>
+      </c>
+      <c r="D6">
+        <v>0.97449168207023995</v>
+      </c>
+      <c r="E6">
+        <v>0.97448597379748603</v>
+      </c>
+      <c r="F6">
+        <v>0.97448661865347397</v>
+      </c>
+      <c r="G6">
+        <v>0.97448550064671102</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="K6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6">
+        <v>0.30421942472457802</v>
+      </c>
+      <c r="M6">
+        <v>0.93956743002544496</v>
+      </c>
+      <c r="N6">
+        <v>0.94067585495322104</v>
+      </c>
+      <c r="O6">
+        <v>0.93956743002544496</v>
+      </c>
+      <c r="P6">
+        <v>0.93977701023206806</v>
+      </c>
+      <c r="Q6">
+        <v>4</v>
+      </c>
+      <c r="T6">
+        <v>20</v>
+      </c>
+      <c r="U6">
+        <v>2.0325217247009202</v>
+      </c>
+      <c r="V6">
+        <v>0.774011299435028</v>
+      </c>
+      <c r="W6">
+        <v>0.77505304633562</v>
+      </c>
+      <c r="X6">
+        <v>0.774011299435028</v>
+      </c>
+      <c r="Y6">
+        <v>0.77443483228985599</v>
+      </c>
+    </row>
+    <row r="7" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B8" s="17"/>
+      <c r="C8" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="20"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="20"/>
+      <c r="T8" s="27">
+        <v>4</v>
+      </c>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19"/>
+      <c r="X8" s="19"/>
+      <c r="Y8" s="20"/>
+    </row>
+    <row r="9" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B9" s="21"/>
+      <c r="H9" s="22"/>
+      <c r="K9" s="21"/>
+      <c r="Q9" s="22"/>
+      <c r="T9" s="21"/>
+      <c r="Y9" s="22"/>
+    </row>
+    <row r="10" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B10" s="21"/>
+      <c r="H10" s="22"/>
+      <c r="K10" s="21"/>
+      <c r="Q10" s="22"/>
+      <c r="T10" s="21"/>
+      <c r="Y10" s="22"/>
+    </row>
+    <row r="11" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B11" s="21"/>
+      <c r="H11" s="22"/>
+      <c r="K11" s="21"/>
+      <c r="Q11" s="22"/>
+      <c r="T11" s="21"/>
+      <c r="Y11" s="22"/>
+    </row>
+    <row r="12" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B12" s="21"/>
+      <c r="H12" s="22"/>
+      <c r="K12" s="21"/>
+      <c r="Q12" s="22"/>
+      <c r="T12" s="21"/>
+      <c r="Y12" s="22"/>
+    </row>
+    <row r="13" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B13" s="21"/>
+      <c r="H13" s="22"/>
+      <c r="K13" s="21"/>
+      <c r="Q13" s="22"/>
+      <c r="T13" s="21"/>
+      <c r="Y13" s="22"/>
+    </row>
+    <row r="14" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B14" s="21"/>
+      <c r="H14" s="22"/>
+      <c r="K14" s="21"/>
+      <c r="Q14" s="22"/>
+      <c r="T14" s="21"/>
+      <c r="Y14" s="22"/>
+    </row>
+    <row r="15" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B15" s="21"/>
+      <c r="H15" s="22"/>
+      <c r="K15" s="21"/>
+      <c r="Q15" s="22"/>
+      <c r="T15" s="21"/>
+      <c r="Y15" s="22"/>
+    </row>
+    <row r="16" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B16" s="21"/>
+      <c r="H16" s="22"/>
+      <c r="K16" s="21"/>
+      <c r="Q16" s="22"/>
+      <c r="T16" s="21"/>
+      <c r="Y16" s="22"/>
+    </row>
+    <row r="17" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B17" s="21"/>
+      <c r="H17" s="22"/>
+      <c r="K17" s="21"/>
+      <c r="Q17" s="22"/>
+      <c r="T17" s="21"/>
+      <c r="Y17" s="22"/>
+    </row>
+    <row r="18" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B18" s="21"/>
+      <c r="H18" s="22"/>
+      <c r="K18" s="21"/>
+      <c r="Q18" s="22"/>
+      <c r="T18" s="21"/>
+      <c r="Y18" s="22"/>
+    </row>
+    <row r="19" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B19" s="21"/>
+      <c r="H19" s="22"/>
+      <c r="K19" s="21"/>
+      <c r="Q19" s="22"/>
+      <c r="T19" s="21"/>
+      <c r="Y19" s="22"/>
+    </row>
+    <row r="20" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B20" s="21"/>
+      <c r="H20" s="22"/>
+      <c r="K20" s="21"/>
+      <c r="Q20" s="22"/>
+      <c r="T20" s="21"/>
+      <c r="Y20" s="22"/>
+    </row>
+    <row r="21" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B21" s="21"/>
+      <c r="H21" s="22"/>
+      <c r="K21" s="21"/>
+      <c r="Q21" s="22"/>
+      <c r="T21" s="21"/>
+      <c r="Y21" s="22"/>
+    </row>
+    <row r="22" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B22" s="21"/>
+      <c r="H22" s="22"/>
+      <c r="K22" s="21"/>
+      <c r="Q22" s="22"/>
+      <c r="T22" s="21"/>
+      <c r="Y22" s="22"/>
+    </row>
+    <row r="23" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B23" s="21"/>
+      <c r="H23" s="22"/>
+      <c r="K23" s="21"/>
+      <c r="Q23" s="22"/>
+      <c r="T23" s="21"/>
+      <c r="Y23" s="22"/>
+    </row>
+    <row r="24" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B24" s="21"/>
+      <c r="H24" s="22"/>
+      <c r="K24" s="21"/>
+      <c r="Q24" s="22"/>
+      <c r="T24" s="21"/>
+      <c r="Y24" s="22"/>
+    </row>
+    <row r="25" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B25" s="21"/>
+      <c r="H25" s="22"/>
+      <c r="K25" s="21"/>
+      <c r="Q25" s="22"/>
+      <c r="T25" s="21"/>
+      <c r="Y25" s="22"/>
+    </row>
+    <row r="26" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B26" s="21"/>
+      <c r="C26" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="H26" s="22"/>
+      <c r="K26" s="21"/>
+      <c r="L26" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="22"/>
+      <c r="T26" s="28">
+        <v>10</v>
+      </c>
+      <c r="Y26" s="22"/>
+    </row>
+    <row r="27" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B27" s="21"/>
+      <c r="H27" s="22"/>
+      <c r="K27" s="21"/>
+      <c r="Q27" s="22"/>
+      <c r="T27" s="21"/>
+      <c r="Y27" s="22"/>
+    </row>
+    <row r="28" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B28" s="21"/>
+      <c r="H28" s="22"/>
+      <c r="K28" s="21"/>
+      <c r="Q28" s="22"/>
+      <c r="T28" s="21"/>
+      <c r="Y28" s="22"/>
+    </row>
+    <row r="29" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B29" s="21"/>
+      <c r="H29" s="22"/>
+      <c r="K29" s="21"/>
+      <c r="Q29" s="22"/>
+      <c r="T29" s="21"/>
+      <c r="Y29" s="22"/>
+    </row>
+    <row r="30" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B30" s="21"/>
+      <c r="H30" s="22"/>
+      <c r="K30" s="21"/>
+      <c r="Q30" s="22"/>
+      <c r="T30" s="21"/>
+      <c r="Y30" s="22"/>
+    </row>
+    <row r="31" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B31" s="21"/>
+      <c r="H31" s="22"/>
+      <c r="K31" s="21"/>
+      <c r="Q31" s="22"/>
+      <c r="T31" s="21"/>
+      <c r="Y31" s="22"/>
+    </row>
+    <row r="32" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B32" s="21"/>
+      <c r="H32" s="22"/>
+      <c r="K32" s="21"/>
+      <c r="Q32" s="22"/>
+      <c r="T32" s="21"/>
+      <c r="Y32" s="22"/>
+    </row>
+    <row r="33" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B33" s="21"/>
+      <c r="H33" s="22"/>
+      <c r="K33" s="21"/>
+      <c r="Q33" s="22"/>
+      <c r="T33" s="21"/>
+      <c r="Y33" s="22"/>
+    </row>
+    <row r="34" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B34" s="21"/>
+      <c r="H34" s="22"/>
+      <c r="K34" s="21"/>
+      <c r="Q34" s="22"/>
+      <c r="T34" s="21"/>
+      <c r="Y34" s="22"/>
+    </row>
+    <row r="35" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B35" s="21"/>
+      <c r="H35" s="22"/>
+      <c r="K35" s="21"/>
+      <c r="Q35" s="22"/>
+      <c r="T35" s="21"/>
+      <c r="Y35" s="22"/>
+    </row>
+    <row r="36" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B36" s="21"/>
+      <c r="H36" s="22"/>
+      <c r="K36" s="21"/>
+      <c r="Q36" s="22"/>
+      <c r="T36" s="21"/>
+      <c r="Y36" s="22"/>
+    </row>
+    <row r="37" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B37" s="21"/>
+      <c r="H37" s="22"/>
+      <c r="K37" s="21"/>
+      <c r="Q37" s="22"/>
+      <c r="T37" s="21"/>
+      <c r="Y37" s="22"/>
+    </row>
+    <row r="38" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B38" s="21"/>
+      <c r="H38" s="22"/>
+      <c r="K38" s="21"/>
+      <c r="Q38" s="22"/>
+      <c r="T38" s="21"/>
+      <c r="Y38" s="22"/>
+    </row>
+    <row r="39" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B39" s="21"/>
+      <c r="H39" s="22"/>
+      <c r="K39" s="21"/>
+      <c r="Q39" s="22"/>
+      <c r="T39" s="21"/>
+      <c r="Y39" s="22"/>
+    </row>
+    <row r="40" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B40" s="21"/>
+      <c r="H40" s="22"/>
+      <c r="K40" s="21"/>
+      <c r="Q40" s="22"/>
+      <c r="T40" s="21"/>
+      <c r="Y40" s="22"/>
+    </row>
+    <row r="41" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B41" s="21"/>
+      <c r="H41" s="22"/>
+      <c r="K41" s="21"/>
+      <c r="Q41" s="22"/>
+      <c r="T41" s="21"/>
+      <c r="Y41" s="22"/>
+    </row>
+    <row r="42" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B42" s="21"/>
+      <c r="H42" s="22"/>
+      <c r="K42" s="21"/>
+      <c r="Q42" s="22"/>
+      <c r="T42" s="21"/>
+      <c r="Y42" s="22"/>
+    </row>
+    <row r="43" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B43" s="21"/>
+      <c r="H43" s="22"/>
+      <c r="K43" s="21"/>
+      <c r="Q43" s="22"/>
+      <c r="T43" s="21"/>
+      <c r="Y43" s="22"/>
+    </row>
+    <row r="44" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B44" s="21"/>
+      <c r="C44" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="H44" s="22"/>
+      <c r="K44" s="21"/>
+      <c r="L44" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q44" s="22"/>
+      <c r="T44" s="28">
+        <v>20</v>
+      </c>
+      <c r="Y44" s="22"/>
+    </row>
+    <row r="45" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B45" s="21"/>
+      <c r="H45" s="22"/>
+      <c r="K45" s="21"/>
+      <c r="Q45" s="22"/>
+      <c r="T45" s="21"/>
+      <c r="Y45" s="22"/>
+    </row>
+    <row r="46" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B46" s="21"/>
+      <c r="H46" s="22"/>
+      <c r="K46" s="21"/>
+      <c r="Q46" s="22"/>
+      <c r="T46" s="21"/>
+      <c r="Y46" s="22"/>
+    </row>
+    <row r="47" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B47" s="21"/>
+      <c r="H47" s="22"/>
+      <c r="K47" s="21"/>
+      <c r="Q47" s="22"/>
+      <c r="T47" s="21"/>
+      <c r="Y47" s="22"/>
+    </row>
+    <row r="48" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B48" s="21"/>
+      <c r="H48" s="22"/>
+      <c r="K48" s="21"/>
+      <c r="Q48" s="22"/>
+      <c r="T48" s="21"/>
+      <c r="Y48" s="22"/>
+    </row>
+    <row r="49" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B49" s="21"/>
+      <c r="H49" s="22"/>
+      <c r="K49" s="21"/>
+      <c r="Q49" s="22"/>
+      <c r="T49" s="21"/>
+      <c r="Y49" s="22"/>
+    </row>
+    <row r="50" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B50" s="21"/>
+      <c r="H50" s="22"/>
+      <c r="K50" s="21"/>
+      <c r="Q50" s="22"/>
+      <c r="T50" s="21"/>
+      <c r="Y50" s="22"/>
+    </row>
+    <row r="51" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B51" s="21"/>
+      <c r="H51" s="22"/>
+      <c r="K51" s="21"/>
+      <c r="Q51" s="22"/>
+      <c r="T51" s="21"/>
+      <c r="Y51" s="22"/>
+    </row>
+    <row r="52" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B52" s="21"/>
+      <c r="H52" s="22"/>
+      <c r="K52" s="21"/>
+      <c r="Q52" s="22"/>
+      <c r="T52" s="21"/>
+      <c r="Y52" s="22"/>
+    </row>
+    <row r="53" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B53" s="21"/>
+      <c r="H53" s="22"/>
+      <c r="K53" s="21"/>
+      <c r="Q53" s="22"/>
+      <c r="T53" s="21"/>
+      <c r="Y53" s="22"/>
+    </row>
+    <row r="54" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B54" s="21"/>
+      <c r="H54" s="22"/>
+      <c r="K54" s="21"/>
+      <c r="Q54" s="22"/>
+      <c r="T54" s="21"/>
+      <c r="Y54" s="22"/>
+    </row>
+    <row r="55" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B55" s="21"/>
+      <c r="H55" s="22"/>
+      <c r="K55" s="21"/>
+      <c r="Q55" s="22"/>
+      <c r="T55" s="21"/>
+      <c r="Y55" s="22"/>
+    </row>
+    <row r="56" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B56" s="21"/>
+      <c r="H56" s="22"/>
+      <c r="K56" s="21"/>
+      <c r="Q56" s="22"/>
+      <c r="T56" s="21"/>
+      <c r="Y56" s="22"/>
+    </row>
+    <row r="57" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B57" s="21"/>
+      <c r="H57" s="22"/>
+      <c r="K57" s="21"/>
+      <c r="Q57" s="22"/>
+      <c r="T57" s="21"/>
+      <c r="Y57" s="22"/>
+    </row>
+    <row r="58" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B58" s="21"/>
+      <c r="H58" s="22"/>
+      <c r="K58" s="21"/>
+      <c r="Q58" s="22"/>
+      <c r="T58" s="21"/>
+      <c r="Y58" s="22"/>
+    </row>
+    <row r="59" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B59" s="21"/>
+      <c r="H59" s="22"/>
+      <c r="K59" s="21"/>
+      <c r="Q59" s="22"/>
+      <c r="T59" s="21"/>
+      <c r="Y59" s="22"/>
+    </row>
+    <row r="60" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B60" s="21"/>
+      <c r="H60" s="22"/>
+      <c r="K60" s="21"/>
+      <c r="Q60" s="22"/>
+      <c r="T60" s="21"/>
+      <c r="Y60" s="22"/>
+    </row>
+    <row r="61" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="24"/>
+      <c r="C61" s="25"/>
+      <c r="D61" s="25"/>
+      <c r="E61" s="25"/>
+      <c r="F61" s="25"/>
+      <c r="G61" s="25"/>
+      <c r="H61" s="26"/>
+      <c r="K61" s="24"/>
+      <c r="L61" s="25"/>
+      <c r="M61" s="25"/>
+      <c r="N61" s="25"/>
+      <c r="O61" s="25"/>
+      <c r="P61" s="25"/>
+      <c r="Q61" s="26"/>
+      <c r="T61" s="21"/>
+      <c r="Y61" s="22"/>
+    </row>
+    <row r="62" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="T62" s="24"/>
+      <c r="U62" s="25"/>
+      <c r="V62" s="25"/>
+      <c r="W62" s="25"/>
+      <c r="X62" s="25"/>
+      <c r="Y62" s="26"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="K2:L2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <tableParts count="3">
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add experiment result from 5th march
</commit_message>
<xml_diff>
--- a/ExperimentsData.xlsx
+++ b/ExperimentsData.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\personal\prethesis-experiments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamchristian/Documents/PersonalProjects/prethesis-experiments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F8A35CE-1806-4A72-B73B-E133120736EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C84AEC4-B60A-EA44-90AC-306BF8DC4898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="3" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="4" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Distribution" sheetId="4" r:id="rId1"/>
     <sheet name="January30th" sheetId="1" r:id="rId2"/>
     <sheet name="February14th" sheetId="2" r:id="rId3"/>
     <sheet name="February25th" sheetId="3" r:id="rId4"/>
+    <sheet name="March5th" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -317,7 +318,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="39">
   <si>
     <t>DistilBERT</t>
   </si>
@@ -428,6 +429,12 @@
   </si>
   <si>
     <t>Indonesian Dataset</t>
+  </si>
+  <si>
+    <t>Epoch 4</t>
+  </si>
+  <si>
+    <t>Epoch 10</t>
   </si>
 </sst>
 </file>
@@ -730,7 +737,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -798,11 +805,43 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="39">
+  <dxfs count="47">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border outline="0">
         <left style="thin">
@@ -1893,6 +1932,99 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>2389</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>745569</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BF77525C-1A17-64C8-8396-67A5816BA670}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="857956" y="3953500"/>
+          <a:ext cx="5389861" cy="3878167"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>42333</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>2714</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>514856</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>183444</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EEA4468F-8CC8-67EA-6940-13E8DADB9601}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7535333" y="3953825"/>
+          <a:ext cx="5467855" cy="3934286"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{306760BC-4A86-48F5-9CF5-A85404614954}" name="Table8" displayName="Table8" ref="B4:C10" totalsRowShown="0">
   <autoFilter ref="B4:C10" xr:uid="{306760BC-4A86-48F5-9CF5-A85404614954}"/>
@@ -1951,11 +2083,26 @@
 </table>
 </file>
 
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{44B3DA9E-56AF-6E4F-B068-8BF057DECD18}" name="Table14" displayName="Table14" ref="B4:G6" totalsRowShown="0" dataDxfId="0" tableBorderDxfId="7">
+  <autoFilter ref="B4:G6" xr:uid="{44B3DA9E-56AF-6E4F-B068-8BF057DECD18}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{A0355691-3CDE-5546-BAEB-FF375EF3AE71}" name="Epoch" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{7C23C618-7B33-934C-A000-84E5D2E16842}" name="Loss" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{1AECA1A5-3BAD-234D-A5A3-B4D822F36581}" name="Accuracy" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{51862FF3-B3FA-734B-A55D-5153C0D2EEE8}" name="Precision" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{60D188E8-68BF-9F45-93D8-4E4338F6C33E}" name="Recall" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{B0F6441D-C47C-F641-A320-DF0003AAAF5E}" name="F1" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{33D6D3E5-9AAF-4914-BE32-298E922BC8A4}" name="Table9" displayName="Table9" ref="B16:C22" totalsRowShown="0">
   <autoFilter ref="B16:C22" xr:uid="{33D6D3E5-9AAF-4914-BE32-298E922BC8A4}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{5155CECE-BBA4-45F8-98E3-DD9D18244FF8}" name="Label" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{5155CECE-BBA4-45F8-98E3-DD9D18244FF8}" name="Label" dataDxfId="46"/>
     <tableColumn id="2" xr3:uid="{6A1175E6-E870-42B6-8AC2-1516761E3F86}" name="Amount"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1963,64 +2110,64 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}" name="Table1" displayName="Table1" ref="B3:H8" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}" name="Table1" displayName="Table1" ref="B3:H8" totalsRowShown="0" headerRowDxfId="45" dataDxfId="44">
   <autoFilter ref="B3:H8" xr:uid="{2E6A850A-6FD6-C847-8F7A-45D1763A074D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{4978B2AE-4B4B-EA49-BF70-5AABACA85971}" name="Dataset Name" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{58D50865-DFF7-8644-AD30-63D47540D02C}" name="Accuracy" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{BBA594A0-A636-D445-AAB9-22C6754D09C0}" name="Precision" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{661E434A-CCB1-BB46-BA1D-8A2D641D7D25}" name="Recall" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{A58BD05A-F5EB-AF4E-A041-498A7ACF41DE}" name="F1" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{B40DA81D-2CB3-F14B-8186-F7D0A18BA0FE}" name="Loss" dataDxfId="30"/>
-    <tableColumn id="7" xr3:uid="{83055B2D-4E00-F845-BC1B-6F22C502B5D2}" name="Epoch" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{4978B2AE-4B4B-EA49-BF70-5AABACA85971}" name="Dataset Name" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{58D50865-DFF7-8644-AD30-63D47540D02C}" name="Accuracy" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{BBA594A0-A636-D445-AAB9-22C6754D09C0}" name="Precision" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{661E434A-CCB1-BB46-BA1D-8A2D641D7D25}" name="Recall" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{A58BD05A-F5EB-AF4E-A041-498A7ACF41DE}" name="F1" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{B40DA81D-2CB3-F14B-8186-F7D0A18BA0FE}" name="Loss" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{83055B2D-4E00-F845-BC1B-6F22C502B5D2}" name="Epoch" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}" name="Table13" displayName="Table13" ref="J12:P18" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}" name="Table13" displayName="Table13" ref="J12:P18" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="J12:P18" xr:uid="{45399445-F25D-ED43-A2D3-36D5D3B280CF}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{EAE6D8E7-8EF0-D94F-A26B-7A025E6C7361}" name="Dataset Name" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{36A28C87-4153-404C-A82A-6C01A5B3DC55}" name="Accuracy" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{E4A45E88-BACC-B941-A1C0-4BBCB2A3CAB7}" name="Precision" dataDxfId="24"/>
-    <tableColumn id="4" xr3:uid="{0106A244-4E6C-994C-8E0B-A39D4088698B}" name="Recall" dataDxfId="23"/>
-    <tableColumn id="5" xr3:uid="{B4A28C88-CF22-604F-982B-A6A1CCF1A1F7}" name="F1" dataDxfId="22"/>
-    <tableColumn id="6" xr3:uid="{0CBF8E57-666D-A545-BA88-90DE39497A4E}" name="Loss" dataDxfId="21"/>
-    <tableColumn id="7" xr3:uid="{944AF69F-9D99-0548-9A49-04236D354F4E}" name="Epoch" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{EAE6D8E7-8EF0-D94F-A26B-7A025E6C7361}" name="Dataset Name" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{36A28C87-4153-404C-A82A-6C01A5B3DC55}" name="Accuracy" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{E4A45E88-BACC-B941-A1C0-4BBCB2A3CAB7}" name="Precision" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{0106A244-4E6C-994C-8E0B-A39D4088698B}" name="Recall" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{B4A28C88-CF22-604F-982B-A6A1CCF1A1F7}" name="F1" dataDxfId="30"/>
+    <tableColumn id="6" xr3:uid="{0CBF8E57-666D-A545-BA88-90DE39497A4E}" name="Loss" dataDxfId="29"/>
+    <tableColumn id="7" xr3:uid="{944AF69F-9D99-0548-9A49-04236D354F4E}" name="Epoch" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}" name="Table134" displayName="Table134" ref="B11:H16" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}" name="Table134" displayName="Table134" ref="B11:H16" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="B11:H16" xr:uid="{148E7717-AEBC-3A4C-9BE3-209010ABE860}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{05A1D84A-55CA-EA40-A483-5E78D383B19B}" name="Dataset Name" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{CA820C5C-5B52-894C-A49F-0549BA14EB14}" name="Accuracy" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{23F3C118-B36A-8344-91C4-91E68C152060}" name="Precision" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{3FDE3D07-7EC9-814A-B04A-1749B565F6EA}" name="Recall" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{4E62075D-7975-3747-9112-6DA05E872576}" name="F1" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{E6B084A9-1443-8E43-8957-DF1E2A9B10B8}" name="Loss" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{AB463B29-B751-9A41-A7DB-1E69264E687D}" name="Epoch" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{05A1D84A-55CA-EA40-A483-5E78D383B19B}" name="Dataset Name" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{CA820C5C-5B52-894C-A49F-0549BA14EB14}" name="Accuracy" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{23F3C118-B36A-8344-91C4-91E68C152060}" name="Precision" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{3FDE3D07-7EC9-814A-B04A-1749B565F6EA}" name="Recall" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{4E62075D-7975-3747-9112-6DA05E872576}" name="F1" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{E6B084A9-1443-8E43-8957-DF1E2A9B10B8}" name="Loss" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{AB463B29-B751-9A41-A7DB-1E69264E687D}" name="Epoch" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}" name="Table7" displayName="Table7" ref="J3:P5" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}" name="Table7" displayName="Table7" ref="J3:P5" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="J3:P5" xr:uid="{3C302D4C-9E14-B546-8FCE-164DCE175359}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{F2E57A4A-2AAD-7447-91C9-007605371819}" name="Model" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{CB02CB06-53A1-2F41-AD51-1547D4DC27A1}" name="Accuracy" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{CA4460C1-43B3-7449-A208-84080D817025}" name="Precision" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{1367CE74-9216-4149-A489-1B4EB4644578}" name="Recall" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{9CF0E2A6-FC0C-744D-AC36-893DD9641356}" name="F1" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{913D2EB3-6EB7-6D45-9EE3-E045E761BD2B}" name="Loss" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{8C15DD0C-3E42-5C44-92F8-BD590893AE2E}" name="Epoch" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{F2E57A4A-2AAD-7447-91C9-007605371819}" name="Model" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{CB02CB06-53A1-2F41-AD51-1547D4DC27A1}" name="Accuracy" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{CA4460C1-43B3-7449-A208-84080D817025}" name="Precision" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{1367CE74-9216-4149-A489-1B4EB4644578}" name="Recall" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{9CF0E2A6-FC0C-744D-AC36-893DD9641356}" name="F1" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{913D2EB3-6EB7-6D45-9EE3-E045E761BD2B}" name="Loss" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{8C15DD0C-3E42-5C44-92F8-BD590893AE2E}" name="Epoch" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2062,7 +2209,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{372BED72-405E-1348-A031-F1B0B5AE3EF5}" name="Table4" displayName="Table4" ref="B19:I23" totalsRowShown="0" headerRowDxfId="1" tableBorderDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{372BED72-405E-1348-A031-F1B0B5AE3EF5}" name="Table4" displayName="Table4" ref="B19:I23" totalsRowShown="0" headerRowDxfId="9" tableBorderDxfId="8">
   <autoFilter ref="B19:I23" xr:uid="{372BED72-405E-1348-A031-F1B0B5AE3EF5}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{1A099EFA-B86F-3A4E-BCA0-D958972A588E}" name="Model"/>
@@ -2396,19 +2543,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F41AEED8-ECB9-41F9-BCFE-8D94D2C04651}">
   <dimension ref="B3:C22"/>
-  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="29" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="29"/>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>23</v>
       </c>
@@ -2416,7 +2563,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>25</v>
       </c>
@@ -2424,7 +2571,7 @@
         <v>5797</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>26</v>
       </c>
@@ -2432,7 +2579,7 @@
         <v>2709</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>27</v>
       </c>
@@ -2440,7 +2587,7 @@
         <v>1641</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>28</v>
       </c>
@@ -2448,7 +2595,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>29</v>
       </c>
@@ -2456,7 +2603,7 @@
         <v>2373</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -2464,13 +2611,13 @@
         <v>6761</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="29" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="29"/>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" t="s">
         <v>23</v>
       </c>
@@ -2478,7 +2625,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" s="16" t="s">
         <v>25</v>
       </c>
@@ -2486,7 +2633,7 @@
         <v>2849</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18" s="15" t="s">
         <v>26</v>
       </c>
@@ -2494,7 +2641,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="16" t="s">
         <v>32</v>
       </c>
@@ -2502,7 +2649,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B20" s="15" t="s">
         <v>28</v>
       </c>
@@ -2510,7 +2657,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B21" s="16" t="s">
         <v>33</v>
       </c>
@@ -2518,7 +2665,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B22" s="15" t="s">
         <v>30</v>
       </c>
@@ -2543,21 +2690,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14964B3B-3353-C742-BCAB-B2A6487822EC}">
   <dimension ref="B2:P19"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.125" style="2"/>
-    <col min="2" max="2" width="28.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.375" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" style="2"/>
+    <col min="2" max="2" width="28.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" style="2" customWidth="1"/>
     <col min="4" max="4" width="10.5" style="2" customWidth="1"/>
-    <col min="5" max="9" width="9.125" style="2"/>
-    <col min="10" max="10" width="24.875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="9" width="9.1640625" style="2"/>
+    <col min="10" max="10" width="24.83203125" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11" style="2" customWidth="1"/>
-    <col min="12" max="12" width="10.875" style="2" customWidth="1"/>
+    <col min="12" max="12" width="10.83203125" style="2" customWidth="1"/>
     <col min="13" max="15" width="10.5" style="2" customWidth="1"/>
-    <col min="16" max="16384" width="9.125" style="2"/>
+    <col min="16" max="16384" width="9.1640625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B2" s="30" t="s">
         <v>0</v>
       </c>
@@ -2566,7 +2713,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -2610,7 +2757,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
@@ -2654,7 +2801,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B5" s="4" t="s">
         <v>12</v>
       </c>
@@ -2698,7 +2845,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
@@ -2721,7 +2868,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B7" s="2" t="s">
         <v>15</v>
       </c>
@@ -2744,7 +2891,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
@@ -2767,13 +2914,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B11" s="2" t="s">
         <v>2</v>
       </c>
@@ -2800,7 +2947,7 @@
       </c>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
@@ -2844,7 +2991,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
@@ -2888,7 +3035,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
@@ -2932,7 +3079,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B15" s="4" t="s">
         <v>12</v>
       </c>
@@ -2976,7 +3123,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B16" s="2" t="s">
         <v>10</v>
       </c>
@@ -3005,7 +3152,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.2">
       <c r="J17" s="2" t="s">
         <v>10</v>
       </c>
@@ -3028,7 +3175,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:C2"/>
@@ -3047,23 +3194,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{480C1162-B378-5D47-92C7-5997231863D1}">
   <dimension ref="B2:I23"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="15.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.375" customWidth="1"/>
+    <col min="2" max="2" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" customWidth="1"/>
     <col min="5" max="5" width="10.5" customWidth="1"/>
     <col min="9" max="9" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B2" s="31" t="s">
         <v>17</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>9</v>
       </c>
@@ -3086,7 +3233,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>11</v>
       </c>
@@ -3109,7 +3256,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>0</v>
       </c>
@@ -3132,7 +3279,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -3155,12 +3302,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>9</v>
       </c>
@@ -3183,7 +3330,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>0</v>
       </c>
@@ -3206,7 +3353,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
         <v>0</v>
       </c>
@@ -3229,7 +3376,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B13" t="s">
         <v>11</v>
       </c>
@@ -3252,7 +3399,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B14" t="s">
         <v>16</v>
       </c>
@@ -3275,7 +3422,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>16</v>
       </c>
@@ -3298,13 +3445,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B18" s="32" t="s">
         <v>19</v>
       </c>
       <c r="C18" s="32"/>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B19" s="8" t="s">
         <v>9</v>
       </c>
@@ -3330,7 +3477,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="11" t="s">
         <v>13</v>
       </c>
@@ -3356,7 +3503,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B21" s="13" t="s">
         <v>13</v>
       </c>
@@ -3382,7 +3529,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
         <v>13</v>
       </c>
@@ -3408,7 +3555,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
         <v>13</v>
       </c>
@@ -3452,10 +3599,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F95E52D2-75E8-D44D-9380-8EC3BF1C86A2}">
   <dimension ref="B1:Y62"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="33" t="s">
         <v>18</v>
       </c>
@@ -3469,7 +3616,7 @@
       </c>
       <c r="U2" s="36"/>
     </row>
-    <row r="3" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>34</v>
       </c>
@@ -3531,7 +3678,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>11</v>
       </c>
@@ -3593,7 +3740,7 @@
         <v>0.77562753371646298</v>
       </c>
     </row>
-    <row r="5" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>0</v>
       </c>
@@ -3655,7 +3802,7 @@
         <v>0.78763665437576802</v>
       </c>
     </row>
-    <row r="6" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -3717,8 +3864,8 @@
         <v>0.77443483228985599</v>
       </c>
     </row>
-    <row r="7" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B8" s="17"/>
       <c r="C8" s="18" t="s">
         <v>11</v>
@@ -3746,7 +3893,7 @@
       <c r="X8" s="19"/>
       <c r="Y8" s="20"/>
     </row>
-    <row r="9" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B9" s="21"/>
       <c r="H9" s="22"/>
       <c r="K9" s="21"/>
@@ -3754,7 +3901,7 @@
       <c r="T9" s="21"/>
       <c r="Y9" s="22"/>
     </row>
-    <row r="10" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B10" s="21"/>
       <c r="H10" s="22"/>
       <c r="K10" s="21"/>
@@ -3762,7 +3909,7 @@
       <c r="T10" s="21"/>
       <c r="Y10" s="22"/>
     </row>
-    <row r="11" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B11" s="21"/>
       <c r="H11" s="22"/>
       <c r="K11" s="21"/>
@@ -3770,7 +3917,7 @@
       <c r="T11" s="21"/>
       <c r="Y11" s="22"/>
     </row>
-    <row r="12" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B12" s="21"/>
       <c r="H12" s="22"/>
       <c r="K12" s="21"/>
@@ -3778,7 +3925,7 @@
       <c r="T12" s="21"/>
       <c r="Y12" s="22"/>
     </row>
-    <row r="13" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B13" s="21"/>
       <c r="H13" s="22"/>
       <c r="K13" s="21"/>
@@ -3786,7 +3933,7 @@
       <c r="T13" s="21"/>
       <c r="Y13" s="22"/>
     </row>
-    <row r="14" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B14" s="21"/>
       <c r="H14" s="22"/>
       <c r="K14" s="21"/>
@@ -3794,7 +3941,7 @@
       <c r="T14" s="21"/>
       <c r="Y14" s="22"/>
     </row>
-    <row r="15" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B15" s="21"/>
       <c r="H15" s="22"/>
       <c r="K15" s="21"/>
@@ -3802,7 +3949,7 @@
       <c r="T15" s="21"/>
       <c r="Y15" s="22"/>
     </row>
-    <row r="16" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B16" s="21"/>
       <c r="H16" s="22"/>
       <c r="K16" s="21"/>
@@ -3810,7 +3957,7 @@
       <c r="T16" s="21"/>
       <c r="Y16" s="22"/>
     </row>
-    <row r="17" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B17" s="21"/>
       <c r="H17" s="22"/>
       <c r="K17" s="21"/>
@@ -3818,7 +3965,7 @@
       <c r="T17" s="21"/>
       <c r="Y17" s="22"/>
     </row>
-    <row r="18" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B18" s="21"/>
       <c r="H18" s="22"/>
       <c r="K18" s="21"/>
@@ -3826,7 +3973,7 @@
       <c r="T18" s="21"/>
       <c r="Y18" s="22"/>
     </row>
-    <row r="19" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B19" s="21"/>
       <c r="H19" s="22"/>
       <c r="K19" s="21"/>
@@ -3834,7 +3981,7 @@
       <c r="T19" s="21"/>
       <c r="Y19" s="22"/>
     </row>
-    <row r="20" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B20" s="21"/>
       <c r="H20" s="22"/>
       <c r="K20" s="21"/>
@@ -3842,7 +3989,7 @@
       <c r="T20" s="21"/>
       <c r="Y20" s="22"/>
     </row>
-    <row r="21" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B21" s="21"/>
       <c r="H21" s="22"/>
       <c r="K21" s="21"/>
@@ -3850,7 +3997,7 @@
       <c r="T21" s="21"/>
       <c r="Y21" s="22"/>
     </row>
-    <row r="22" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B22" s="21"/>
       <c r="H22" s="22"/>
       <c r="K22" s="21"/>
@@ -3858,7 +4005,7 @@
       <c r="T22" s="21"/>
       <c r="Y22" s="22"/>
     </row>
-    <row r="23" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B23" s="21"/>
       <c r="H23" s="22"/>
       <c r="K23" s="21"/>
@@ -3866,7 +4013,7 @@
       <c r="T23" s="21"/>
       <c r="Y23" s="22"/>
     </row>
-    <row r="24" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B24" s="21"/>
       <c r="H24" s="22"/>
       <c r="K24" s="21"/>
@@ -3874,7 +4021,7 @@
       <c r="T24" s="21"/>
       <c r="Y24" s="22"/>
     </row>
-    <row r="25" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B25" s="21"/>
       <c r="H25" s="22"/>
       <c r="K25" s="21"/>
@@ -3882,7 +4029,7 @@
       <c r="T25" s="21"/>
       <c r="Y25" s="22"/>
     </row>
-    <row r="26" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B26" s="21"/>
       <c r="C26" s="23" t="s">
         <v>0</v>
@@ -3898,7 +4045,7 @@
       </c>
       <c r="Y26" s="22"/>
     </row>
-    <row r="27" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B27" s="21"/>
       <c r="H27" s="22"/>
       <c r="K27" s="21"/>
@@ -3906,7 +4053,7 @@
       <c r="T27" s="21"/>
       <c r="Y27" s="22"/>
     </row>
-    <row r="28" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B28" s="21"/>
       <c r="H28" s="22"/>
       <c r="K28" s="21"/>
@@ -3914,7 +4061,7 @@
       <c r="T28" s="21"/>
       <c r="Y28" s="22"/>
     </row>
-    <row r="29" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B29" s="21"/>
       <c r="H29" s="22"/>
       <c r="K29" s="21"/>
@@ -3922,7 +4069,7 @@
       <c r="T29" s="21"/>
       <c r="Y29" s="22"/>
     </row>
-    <row r="30" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B30" s="21"/>
       <c r="H30" s="22"/>
       <c r="K30" s="21"/>
@@ -3930,7 +4077,7 @@
       <c r="T30" s="21"/>
       <c r="Y30" s="22"/>
     </row>
-    <row r="31" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B31" s="21"/>
       <c r="H31" s="22"/>
       <c r="K31" s="21"/>
@@ -3938,7 +4085,7 @@
       <c r="T31" s="21"/>
       <c r="Y31" s="22"/>
     </row>
-    <row r="32" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B32" s="21"/>
       <c r="H32" s="22"/>
       <c r="K32" s="21"/>
@@ -3946,7 +4093,7 @@
       <c r="T32" s="21"/>
       <c r="Y32" s="22"/>
     </row>
-    <row r="33" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B33" s="21"/>
       <c r="H33" s="22"/>
       <c r="K33" s="21"/>
@@ -3954,7 +4101,7 @@
       <c r="T33" s="21"/>
       <c r="Y33" s="22"/>
     </row>
-    <row r="34" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B34" s="21"/>
       <c r="H34" s="22"/>
       <c r="K34" s="21"/>
@@ -3962,7 +4109,7 @@
       <c r="T34" s="21"/>
       <c r="Y34" s="22"/>
     </row>
-    <row r="35" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B35" s="21"/>
       <c r="H35" s="22"/>
       <c r="K35" s="21"/>
@@ -3970,7 +4117,7 @@
       <c r="T35" s="21"/>
       <c r="Y35" s="22"/>
     </row>
-    <row r="36" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B36" s="21"/>
       <c r="H36" s="22"/>
       <c r="K36" s="21"/>
@@ -3978,7 +4125,7 @@
       <c r="T36" s="21"/>
       <c r="Y36" s="22"/>
     </row>
-    <row r="37" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B37" s="21"/>
       <c r="H37" s="22"/>
       <c r="K37" s="21"/>
@@ -3986,7 +4133,7 @@
       <c r="T37" s="21"/>
       <c r="Y37" s="22"/>
     </row>
-    <row r="38" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B38" s="21"/>
       <c r="H38" s="22"/>
       <c r="K38" s="21"/>
@@ -3994,7 +4141,7 @@
       <c r="T38" s="21"/>
       <c r="Y38" s="22"/>
     </row>
-    <row r="39" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B39" s="21"/>
       <c r="H39" s="22"/>
       <c r="K39" s="21"/>
@@ -4002,7 +4149,7 @@
       <c r="T39" s="21"/>
       <c r="Y39" s="22"/>
     </row>
-    <row r="40" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B40" s="21"/>
       <c r="H40" s="22"/>
       <c r="K40" s="21"/>
@@ -4010,7 +4157,7 @@
       <c r="T40" s="21"/>
       <c r="Y40" s="22"/>
     </row>
-    <row r="41" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B41" s="21"/>
       <c r="H41" s="22"/>
       <c r="K41" s="21"/>
@@ -4018,7 +4165,7 @@
       <c r="T41" s="21"/>
       <c r="Y41" s="22"/>
     </row>
-    <row r="42" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B42" s="21"/>
       <c r="H42" s="22"/>
       <c r="K42" s="21"/>
@@ -4026,7 +4173,7 @@
       <c r="T42" s="21"/>
       <c r="Y42" s="22"/>
     </row>
-    <row r="43" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B43" s="21"/>
       <c r="H43" s="22"/>
       <c r="K43" s="21"/>
@@ -4034,7 +4181,7 @@
       <c r="T43" s="21"/>
       <c r="Y43" s="22"/>
     </row>
-    <row r="44" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B44" s="21"/>
       <c r="C44" s="23" t="s">
         <v>16</v>
@@ -4050,7 +4197,7 @@
       </c>
       <c r="Y44" s="22"/>
     </row>
-    <row r="45" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B45" s="21"/>
       <c r="H45" s="22"/>
       <c r="K45" s="21"/>
@@ -4058,7 +4205,7 @@
       <c r="T45" s="21"/>
       <c r="Y45" s="22"/>
     </row>
-    <row r="46" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B46" s="21"/>
       <c r="H46" s="22"/>
       <c r="K46" s="21"/>
@@ -4066,7 +4213,7 @@
       <c r="T46" s="21"/>
       <c r="Y46" s="22"/>
     </row>
-    <row r="47" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B47" s="21"/>
       <c r="H47" s="22"/>
       <c r="K47" s="21"/>
@@ -4074,7 +4221,7 @@
       <c r="T47" s="21"/>
       <c r="Y47" s="22"/>
     </row>
-    <row r="48" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B48" s="21"/>
       <c r="H48" s="22"/>
       <c r="K48" s="21"/>
@@ -4082,7 +4229,7 @@
       <c r="T48" s="21"/>
       <c r="Y48" s="22"/>
     </row>
-    <row r="49" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B49" s="21"/>
       <c r="H49" s="22"/>
       <c r="K49" s="21"/>
@@ -4090,7 +4237,7 @@
       <c r="T49" s="21"/>
       <c r="Y49" s="22"/>
     </row>
-    <row r="50" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B50" s="21"/>
       <c r="H50" s="22"/>
       <c r="K50" s="21"/>
@@ -4098,7 +4245,7 @@
       <c r="T50" s="21"/>
       <c r="Y50" s="22"/>
     </row>
-    <row r="51" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B51" s="21"/>
       <c r="H51" s="22"/>
       <c r="K51" s="21"/>
@@ -4106,7 +4253,7 @@
       <c r="T51" s="21"/>
       <c r="Y51" s="22"/>
     </row>
-    <row r="52" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B52" s="21"/>
       <c r="H52" s="22"/>
       <c r="K52" s="21"/>
@@ -4114,7 +4261,7 @@
       <c r="T52" s="21"/>
       <c r="Y52" s="22"/>
     </row>
-    <row r="53" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B53" s="21"/>
       <c r="H53" s="22"/>
       <c r="K53" s="21"/>
@@ -4122,7 +4269,7 @@
       <c r="T53" s="21"/>
       <c r="Y53" s="22"/>
     </row>
-    <row r="54" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B54" s="21"/>
       <c r="H54" s="22"/>
       <c r="K54" s="21"/>
@@ -4130,7 +4277,7 @@
       <c r="T54" s="21"/>
       <c r="Y54" s="22"/>
     </row>
-    <row r="55" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B55" s="21"/>
       <c r="H55" s="22"/>
       <c r="K55" s="21"/>
@@ -4138,7 +4285,7 @@
       <c r="T55" s="21"/>
       <c r="Y55" s="22"/>
     </row>
-    <row r="56" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B56" s="21"/>
       <c r="H56" s="22"/>
       <c r="K56" s="21"/>
@@ -4146,7 +4293,7 @@
       <c r="T56" s="21"/>
       <c r="Y56" s="22"/>
     </row>
-    <row r="57" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B57" s="21"/>
       <c r="H57" s="22"/>
       <c r="K57" s="21"/>
@@ -4154,7 +4301,7 @@
       <c r="T57" s="21"/>
       <c r="Y57" s="22"/>
     </row>
-    <row r="58" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B58" s="21"/>
       <c r="H58" s="22"/>
       <c r="K58" s="21"/>
@@ -4162,7 +4309,7 @@
       <c r="T58" s="21"/>
       <c r="Y58" s="22"/>
     </row>
-    <row r="59" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B59" s="21"/>
       <c r="H59" s="22"/>
       <c r="K59" s="21"/>
@@ -4170,7 +4317,7 @@
       <c r="T59" s="21"/>
       <c r="Y59" s="22"/>
     </row>
-    <row r="60" spans="2:25" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:25" x14ac:dyDescent="0.2">
       <c r="B60" s="21"/>
       <c r="H60" s="22"/>
       <c r="K60" s="21"/>
@@ -4178,7 +4325,7 @@
       <c r="T60" s="21"/>
       <c r="Y60" s="22"/>
     </row>
-    <row r="61" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B61" s="24"/>
       <c r="C61" s="25"/>
       <c r="D61" s="25"/>
@@ -4196,7 +4343,7 @@
       <c r="T61" s="21"/>
       <c r="Y61" s="22"/>
     </row>
-    <row r="62" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="T62" s="24"/>
       <c r="U62" s="25"/>
       <c r="V62" s="25"/>
@@ -4219,4 +4366,96 @@
     <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F4196E-D435-064A-B41B-979B9B2AEE8B}">
+  <dimension ref="B3:J20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="17.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="38">
+        <v>4</v>
+      </c>
+      <c r="C5" s="37">
+        <v>1.0810999999999999</v>
+      </c>
+      <c r="D5" s="37">
+        <v>0.75480199999999997</v>
+      </c>
+      <c r="E5" s="37">
+        <v>0.75643000000000005</v>
+      </c>
+      <c r="F5" s="37">
+        <v>0.75480199999999997</v>
+      </c>
+      <c r="G5" s="39">
+        <v>0.75505</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="40">
+        <v>10</v>
+      </c>
+      <c r="C6" s="40">
+        <v>1.7057</v>
+      </c>
+      <c r="D6" s="40">
+        <v>0.76384099999999999</v>
+      </c>
+      <c r="E6" s="40">
+        <v>0.76824000000000003</v>
+      </c>
+      <c r="F6" s="40">
+        <v>0.76383999999999996</v>
+      </c>
+      <c r="G6" s="40">
+        <v>0.76429000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="J20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add experiments results
</commit_message>
<xml_diff>
--- a/ExperimentsData.xlsx
+++ b/ExperimentsData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/williamchristian/Documents/PersonalProjects/prethesis-experiments/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GithubProjects\prethesis-experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C84AEC4-B60A-EA44-90AC-306BF8DC4898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{536C8710-A5A5-44B0-9A23-532120AD738D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="4" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="5" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Distribution" sheetId="4" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="February14th" sheetId="2" r:id="rId3"/>
     <sheet name="February25th" sheetId="3" r:id="rId4"/>
     <sheet name="March5th" sheetId="5" r:id="rId5"/>
+    <sheet name="March11th" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -318,7 +319,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="147">
   <si>
     <t>DistilBERT</t>
   </si>
@@ -435,6 +436,330 @@
   </si>
   <si>
     <t>Epoch 10</t>
+  </si>
+  <si>
+    <t>dataset</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>epochs</t>
+  </si>
+  <si>
+    <t>dropout</t>
+  </si>
+  <si>
+    <t>learning_rate</t>
+  </si>
+  <si>
+    <t>weight_decay</t>
+  </si>
+  <si>
+    <t>early_stopping</t>
+  </si>
+  <si>
+    <t>batch_size</t>
+  </si>
+  <si>
+    <t>eval_loss</t>
+  </si>
+  <si>
+    <t>eval_accuracy</t>
+  </si>
+  <si>
+    <t>eval_precision</t>
+  </si>
+  <si>
+    <t>eval_recall</t>
+  </si>
+  <si>
+    <t>eval_f1</t>
+  </si>
+  <si>
+    <t>eval_runtime</t>
+  </si>
+  <si>
+    <t>eval_samples_per_second</t>
+  </si>
+  <si>
+    <t>eval_steps_per_second</t>
+  </si>
+  <si>
+    <t>epoch</t>
+  </si>
+  <si>
+    <t>IndonesiaDataset</t>
+  </si>
+  <si>
+    <t>model-AptaArkana-indonesian-distilbert-base-cased-finetuned-indonlu</t>
+  </si>
+  <si>
+    <t>0.9020816683769226</t>
+  </si>
+  <si>
+    <t>0.7412429378531074</t>
+  </si>
+  <si>
+    <t>0.7437560879084091</t>
+  </si>
+  <si>
+    <t>0.7412429378531072</t>
+  </si>
+  <si>
+    <t>0.7412125065843697</t>
+  </si>
+  <si>
+    <t>9.957110609480813</t>
+  </si>
+  <si>
+    <t>1.3217127323150635</t>
+  </si>
+  <si>
+    <t>0.7435028248587571</t>
+  </si>
+  <si>
+    <t>0.7459095873478361</t>
+  </si>
+  <si>
+    <t>0.7432972198757353</t>
+  </si>
+  <si>
+    <t>9.978531073446328</t>
+  </si>
+  <si>
+    <t>0.7144429678848283</t>
+  </si>
+  <si>
+    <t>0.7118644067796609</t>
+  </si>
+  <si>
+    <t>0.7125270885601606</t>
+  </si>
+  <si>
+    <t>1.3187475204467773</t>
+  </si>
+  <si>
+    <t>0.7543174516602263</t>
+  </si>
+  <si>
+    <t>0.7511781055977554</t>
+  </si>
+  <si>
+    <t>1.3306825160980225</t>
+  </si>
+  <si>
+    <t>0.7468926553672316</t>
+  </si>
+  <si>
+    <t>0.7494229911063286</t>
+  </si>
+  <si>
+    <t>0.7468926553672317</t>
+  </si>
+  <si>
+    <t>0.7467158526700747</t>
+  </si>
+  <si>
+    <t>0.7677558660507202</t>
+  </si>
+  <si>
+    <t>0.7028248587570621</t>
+  </si>
+  <si>
+    <t>0.7047540777421412</t>
+  </si>
+  <si>
+    <t>0.7028248587570622</t>
+  </si>
+  <si>
+    <t>4.979683972911964</t>
+  </si>
+  <si>
+    <t>0.7997637391090393</t>
+  </si>
+  <si>
+    <t>0.7344632768361582</t>
+  </si>
+  <si>
+    <t>0.7344632768361581</t>
+  </si>
+  <si>
+    <t>0.7347434778036733</t>
+  </si>
+  <si>
+    <t>4.989830508474577</t>
+  </si>
+  <si>
+    <t>0.8001335263252258</t>
+  </si>
+  <si>
+    <t>0.7299435028248588</t>
+  </si>
+  <si>
+    <t>0.7349090257515583</t>
+  </si>
+  <si>
+    <t>0.7299435028248586</t>
+  </si>
+  <si>
+    <t>0.7302405658535566</t>
+  </si>
+  <si>
+    <t>0.6734463276836158</t>
+  </si>
+  <si>
+    <t>0.6792741672563136</t>
+  </si>
+  <si>
+    <t>0.6730737753267759</t>
+  </si>
+  <si>
+    <t>0.8017615079879761</t>
+  </si>
+  <si>
+    <t>0.7333333333333333</t>
+  </si>
+  <si>
+    <t>0.7990424633026123</t>
+  </si>
+  <si>
+    <t>0.7400028039028257</t>
+  </si>
+  <si>
+    <t>0.7358274886437817</t>
+  </si>
+  <si>
+    <t>model-indobenchmark-indobert-base-p1</t>
+  </si>
+  <si>
+    <t>1.1265259981155396</t>
+  </si>
+  <si>
+    <t>0.7966101694915254</t>
+  </si>
+  <si>
+    <t>0.7979455731806371</t>
+  </si>
+  <si>
+    <t>0.7970311391291125</t>
+  </si>
+  <si>
+    <t>1.3319859504699707</t>
+  </si>
+  <si>
+    <t>0.7864406779661017</t>
+  </si>
+  <si>
+    <t>0.7897225747196608</t>
+  </si>
+  <si>
+    <t>0.7866627356385301</t>
+  </si>
+  <si>
+    <t>1.266667366027832</t>
+  </si>
+  <si>
+    <t>0.8007303795035394</t>
+  </si>
+  <si>
+    <t>0.9782410264015198</t>
+  </si>
+  <si>
+    <t>0.7887005649717514</t>
+  </si>
+  <si>
+    <t>0.7925478409952664</t>
+  </si>
+  <si>
+    <t>0.7887005649717513</t>
+  </si>
+  <si>
+    <t>0.7892754945297147</t>
+  </si>
+  <si>
+    <t>1.3446446657180786</t>
+  </si>
+  <si>
+    <t>0.7909752913667181</t>
+  </si>
+  <si>
+    <t>0.7864406779661016</t>
+  </si>
+  <si>
+    <t>0.7872570814586577</t>
+  </si>
+  <si>
+    <t>1.2965186834335327</t>
+  </si>
+  <si>
+    <t>0.7932203389830509</t>
+  </si>
+  <si>
+    <t>0.7982197797684893</t>
+  </si>
+  <si>
+    <t>0.7938507297068459</t>
+  </si>
+  <si>
+    <t>0.7491408586502075</t>
+  </si>
+  <si>
+    <t>0.7819209039548023</t>
+  </si>
+  <si>
+    <t>0.7866572045858558</t>
+  </si>
+  <si>
+    <t>0.7823852956530034</t>
+  </si>
+  <si>
+    <t>0.9590385556221008</t>
+  </si>
+  <si>
+    <t>0.7830508474576271</t>
+  </si>
+  <si>
+    <t>0.7830508474576272</t>
+  </si>
+  <si>
+    <t>0.7838155597372222</t>
+  </si>
+  <si>
+    <t>0.9632648229598999</t>
+  </si>
+  <si>
+    <t>0.7875706214689265</t>
+  </si>
+  <si>
+    <t>0.7912551460704853</t>
+  </si>
+  <si>
+    <t>0.7875706214689264</t>
+  </si>
+  <si>
+    <t>0.7879377767489796</t>
+  </si>
+  <si>
+    <t>0.6486183404922485</t>
+  </si>
+  <si>
+    <t>0.7694915254237288</t>
+  </si>
+  <si>
+    <t>0.7699342643018308</t>
+  </si>
+  <si>
+    <t>0.9695460200309753</t>
+  </si>
+  <si>
+    <t>0.7893925977836567</t>
+  </si>
+  <si>
+    <t>0.7868278618140787</t>
+  </si>
+  <si>
+    <t>0.9695459604263306</t>
   </si>
 </sst>
 </file>
@@ -737,7 +1062,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -805,10 +1130,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -833,14 +1155,14 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <border outline="0">
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -2084,15 +2406,41 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{44B3DA9E-56AF-6E4F-B068-8BF057DECD18}" name="Table14" displayName="Table14" ref="B4:G6" totalsRowShown="0" dataDxfId="0" tableBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{44B3DA9E-56AF-6E4F-B068-8BF057DECD18}" name="Table14" displayName="Table14" ref="B4:G6" totalsRowShown="0" dataDxfId="7" tableBorderDxfId="6">
   <autoFilter ref="B4:G6" xr:uid="{44B3DA9E-56AF-6E4F-B068-8BF057DECD18}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{A0355691-3CDE-5546-BAEB-FF375EF3AE71}" name="Epoch" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{7C23C618-7B33-934C-A000-84E5D2E16842}" name="Loss" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{1AECA1A5-3BAD-234D-A5A3-B4D822F36581}" name="Accuracy" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{51862FF3-B3FA-734B-A55D-5153C0D2EEE8}" name="Precision" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{60D188E8-68BF-9F45-93D8-4E4338F6C33E}" name="Recall" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{B0F6441D-C47C-F641-A320-DF0003AAAF5E}" name="F1" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{A0355691-3CDE-5546-BAEB-FF375EF3AE71}" name="Epoch" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{7C23C618-7B33-934C-A000-84E5D2E16842}" name="Loss" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{1AECA1A5-3BAD-234D-A5A3-B4D822F36581}" name="Accuracy" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{51862FF3-B3FA-734B-A55D-5153C0D2EEE8}" name="Precision" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{60D188E8-68BF-9F45-93D8-4E4338F6C33E}" name="Recall" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{B0F6441D-C47C-F641-A320-DF0003AAAF5E}" name="F1" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{0BE9469F-19B5-434A-A19E-F3BD96A4DB2E}" name="Table15" displayName="Table15" ref="A1:Q24" totalsRowShown="0">
+  <autoFilter ref="A1:Q24" xr:uid="{0BE9469F-19B5-434A-A19E-F3BD96A4DB2E}"/>
+  <tableColumns count="17">
+    <tableColumn id="1" xr3:uid="{F0238EF6-C541-4B95-81D7-4EC51722F2C5}" name="dataset"/>
+    <tableColumn id="2" xr3:uid="{7FFF71A5-DBF2-4BDC-8A6B-F6EFFF3F7726}" name="model"/>
+    <tableColumn id="3" xr3:uid="{F79AAD39-55FA-4924-801E-996B2A7BCA5C}" name="epochs"/>
+    <tableColumn id="4" xr3:uid="{2E64B84D-B204-4142-9DF8-BD89D6311791}" name="dropout"/>
+    <tableColumn id="5" xr3:uid="{430D06A4-2618-4E0D-BE51-7C49D1264119}" name="learning_rate"/>
+    <tableColumn id="6" xr3:uid="{89A160B3-7852-4287-8EB0-1BFD5B8C26F5}" name="weight_decay"/>
+    <tableColumn id="7" xr3:uid="{E5BDEE13-693F-417F-A34F-6B17F62DF5E9}" name="early_stopping"/>
+    <tableColumn id="8" xr3:uid="{B81F4116-A6E8-46AE-B9ED-9E73C0631A05}" name="batch_size"/>
+    <tableColumn id="9" xr3:uid="{42A43892-BB90-41BD-A46D-0AE680CAFC46}" name="eval_loss"/>
+    <tableColumn id="10" xr3:uid="{5D3ADF4C-E2EB-4AC9-B3A2-26E4CE07B46B}" name="eval_accuracy"/>
+    <tableColumn id="11" xr3:uid="{4687ACB0-D0AF-49FA-BFFD-73772299764A}" name="eval_precision"/>
+    <tableColumn id="12" xr3:uid="{5FB6D644-FEF0-40D8-AEAD-2CB00158C852}" name="eval_recall"/>
+    <tableColumn id="13" xr3:uid="{4EB7C555-9212-4DD7-806C-AD747CD6C46B}" name="eval_f1"/>
+    <tableColumn id="14" xr3:uid="{B358371A-77CC-4489-9FA7-7129AD5AB5EA}" name="eval_runtime"/>
+    <tableColumn id="15" xr3:uid="{B27A0A83-E411-4CEE-80A4-0D7B5E67FA44}" name="eval_samples_per_second"/>
+    <tableColumn id="16" xr3:uid="{9E98B6F5-5B14-4F59-B65B-7B65970D6E99}" name="eval_steps_per_second"/>
+    <tableColumn id="17" xr3:uid="{7347B754-27FE-4933-B2FF-A25A3E7D63D4}" name="epoch"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2543,19 +2891,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F41AEED8-ECB9-41F9-BCFE-8D94D2C04651}">
   <dimension ref="B3:C22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="29" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="29"/>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>23</v>
       </c>
@@ -2563,7 +2911,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>25</v>
       </c>
@@ -2571,7 +2919,7 @@
         <v>5797</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>26</v>
       </c>
@@ -2579,7 +2927,7 @@
         <v>2709</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>27</v>
       </c>
@@ -2587,7 +2935,7 @@
         <v>1641</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>28</v>
       </c>
@@ -2595,7 +2943,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>29</v>
       </c>
@@ -2603,7 +2951,7 @@
         <v>2373</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>30</v>
       </c>
@@ -2611,13 +2959,13 @@
         <v>6761</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15" s="29" t="s">
         <v>31</v>
       </c>
       <c r="C15" s="29"/>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>23</v>
       </c>
@@ -2625,7 +2973,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="16" t="s">
         <v>25</v>
       </c>
@@ -2633,7 +2981,7 @@
         <v>2849</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="15" t="s">
         <v>26</v>
       </c>
@@ -2641,7 +2989,7 @@
         <v>1341</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="16" t="s">
         <v>32</v>
       </c>
@@ -2649,7 +2997,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" s="15" t="s">
         <v>28</v>
       </c>
@@ -2657,7 +3005,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21" s="16" t="s">
         <v>33</v>
       </c>
@@ -2665,7 +3013,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B22" s="15" t="s">
         <v>30</v>
       </c>
@@ -2690,21 +3038,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14964B3B-3353-C742-BCAB-B2A6487822EC}">
   <dimension ref="B2:P19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="2"/>
-    <col min="2" max="2" width="28.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9.125" style="2"/>
+    <col min="2" max="2" width="28.375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.375" style="2" customWidth="1"/>
     <col min="4" max="4" width="10.5" style="2" customWidth="1"/>
-    <col min="5" max="9" width="9.1640625" style="2"/>
-    <col min="10" max="10" width="24.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="9" width="9.125" style="2"/>
+    <col min="10" max="10" width="24.875" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11" style="2" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" style="2" customWidth="1"/>
+    <col min="12" max="12" width="10.875" style="2" customWidth="1"/>
     <col min="13" max="15" width="10.5" style="2" customWidth="1"/>
-    <col min="16" max="16384" width="9.1640625" style="2"/>
+    <col min="16" max="16384" width="9.125" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B2" s="30" t="s">
         <v>0</v>
       </c>
@@ -2713,7 +3061,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -2757,7 +3105,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
@@ -2801,7 +3149,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>12</v>
       </c>
@@ -2845,7 +3193,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
@@ -2868,7 +3216,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>15</v>
       </c>
@@ -2891,7 +3239,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
@@ -2914,13 +3262,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="1"/>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
         <v>2</v>
       </c>
@@ -2947,7 +3295,7 @@
       </c>
       <c r="K11" s="1"/>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
         <v>10</v>
       </c>
@@ -2991,7 +3339,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
@@ -3035,7 +3383,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
@@ -3079,7 +3427,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
         <v>12</v>
       </c>
@@ -3123,7 +3471,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>10</v>
       </c>
@@ -3152,7 +3500,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="J17" s="2" t="s">
         <v>10</v>
       </c>
@@ -3175,7 +3523,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:C2"/>
@@ -3194,23 +3542,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{480C1162-B378-5D47-92C7-5997231863D1}">
   <dimension ref="B2:I23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.375" customWidth="1"/>
     <col min="5" max="5" width="10.5" customWidth="1"/>
     <col min="9" max="9" width="17.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="31" t="s">
         <v>17</v>
       </c>
       <c r="C2" s="31"/>
       <c r="D2" s="31"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>9</v>
       </c>
@@ -3233,7 +3581,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>11</v>
       </c>
@@ -3256,7 +3604,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>0</v>
       </c>
@@ -3279,7 +3627,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -3302,12 +3650,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>9</v>
       </c>
@@ -3330,7 +3678,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>0</v>
       </c>
@@ -3353,7 +3701,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>0</v>
       </c>
@@ -3376,7 +3724,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>11</v>
       </c>
@@ -3399,7 +3747,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>16</v>
       </c>
@@ -3422,7 +3770,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>16</v>
       </c>
@@ -3445,13 +3793,13 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B18" s="32" t="s">
         <v>19</v>
       </c>
       <c r="C18" s="32"/>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="8" t="s">
         <v>9</v>
       </c>
@@ -3477,7 +3825,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="11" t="s">
         <v>13</v>
       </c>
@@ -3503,7 +3851,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="13" t="s">
         <v>13</v>
       </c>
@@ -3529,7 +3877,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>13</v>
       </c>
@@ -3555,7 +3903,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>13</v>
       </c>
@@ -3599,10 +3947,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F95E52D2-75E8-D44D-9380-8EC3BF1C86A2}">
   <dimension ref="B1:Y62"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="33" t="s">
         <v>18</v>
       </c>
@@ -3616,7 +3964,7 @@
       </c>
       <c r="U2" s="36"/>
     </row>
-    <row r="3" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>34</v>
       </c>
@@ -3678,7 +4026,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>11</v>
       </c>
@@ -3740,7 +4088,7 @@
         <v>0.77562753371646298</v>
       </c>
     </row>
-    <row r="5" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>0</v>
       </c>
@@ -3802,7 +4150,7 @@
         <v>0.78763665437576802</v>
       </c>
     </row>
-    <row r="6" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>16</v>
       </c>
@@ -3864,8 +4212,8 @@
         <v>0.77443483228985599</v>
       </c>
     </row>
-    <row r="7" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B8" s="17"/>
       <c r="C8" s="18" t="s">
         <v>11</v>
@@ -3893,7 +4241,7 @@
       <c r="X8" s="19"/>
       <c r="Y8" s="20"/>
     </row>
-    <row r="9" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B9" s="21"/>
       <c r="H9" s="22"/>
       <c r="K9" s="21"/>
@@ -3901,7 +4249,7 @@
       <c r="T9" s="21"/>
       <c r="Y9" s="22"/>
     </row>
-    <row r="10" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B10" s="21"/>
       <c r="H10" s="22"/>
       <c r="K10" s="21"/>
@@ -3909,7 +4257,7 @@
       <c r="T10" s="21"/>
       <c r="Y10" s="22"/>
     </row>
-    <row r="11" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B11" s="21"/>
       <c r="H11" s="22"/>
       <c r="K11" s="21"/>
@@ -3917,7 +4265,7 @@
       <c r="T11" s="21"/>
       <c r="Y11" s="22"/>
     </row>
-    <row r="12" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B12" s="21"/>
       <c r="H12" s="22"/>
       <c r="K12" s="21"/>
@@ -3925,7 +4273,7 @@
       <c r="T12" s="21"/>
       <c r="Y12" s="22"/>
     </row>
-    <row r="13" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B13" s="21"/>
       <c r="H13" s="22"/>
       <c r="K13" s="21"/>
@@ -3933,7 +4281,7 @@
       <c r="T13" s="21"/>
       <c r="Y13" s="22"/>
     </row>
-    <row r="14" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B14" s="21"/>
       <c r="H14" s="22"/>
       <c r="K14" s="21"/>
@@ -3941,7 +4289,7 @@
       <c r="T14" s="21"/>
       <c r="Y14" s="22"/>
     </row>
-    <row r="15" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B15" s="21"/>
       <c r="H15" s="22"/>
       <c r="K15" s="21"/>
@@ -3949,7 +4297,7 @@
       <c r="T15" s="21"/>
       <c r="Y15" s="22"/>
     </row>
-    <row r="16" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B16" s="21"/>
       <c r="H16" s="22"/>
       <c r="K16" s="21"/>
@@ -3957,7 +4305,7 @@
       <c r="T16" s="21"/>
       <c r="Y16" s="22"/>
     </row>
-    <row r="17" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B17" s="21"/>
       <c r="H17" s="22"/>
       <c r="K17" s="21"/>
@@ -3965,7 +4313,7 @@
       <c r="T17" s="21"/>
       <c r="Y17" s="22"/>
     </row>
-    <row r="18" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B18" s="21"/>
       <c r="H18" s="22"/>
       <c r="K18" s="21"/>
@@ -3973,7 +4321,7 @@
       <c r="T18" s="21"/>
       <c r="Y18" s="22"/>
     </row>
-    <row r="19" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B19" s="21"/>
       <c r="H19" s="22"/>
       <c r="K19" s="21"/>
@@ -3981,7 +4329,7 @@
       <c r="T19" s="21"/>
       <c r="Y19" s="22"/>
     </row>
-    <row r="20" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B20" s="21"/>
       <c r="H20" s="22"/>
       <c r="K20" s="21"/>
@@ -3989,7 +4337,7 @@
       <c r="T20" s="21"/>
       <c r="Y20" s="22"/>
     </row>
-    <row r="21" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B21" s="21"/>
       <c r="H21" s="22"/>
       <c r="K21" s="21"/>
@@ -3997,7 +4345,7 @@
       <c r="T21" s="21"/>
       <c r="Y21" s="22"/>
     </row>
-    <row r="22" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B22" s="21"/>
       <c r="H22" s="22"/>
       <c r="K22" s="21"/>
@@ -4005,7 +4353,7 @@
       <c r="T22" s="21"/>
       <c r="Y22" s="22"/>
     </row>
-    <row r="23" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B23" s="21"/>
       <c r="H23" s="22"/>
       <c r="K23" s="21"/>
@@ -4013,7 +4361,7 @@
       <c r="T23" s="21"/>
       <c r="Y23" s="22"/>
     </row>
-    <row r="24" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B24" s="21"/>
       <c r="H24" s="22"/>
       <c r="K24" s="21"/>
@@ -4021,7 +4369,7 @@
       <c r="T24" s="21"/>
       <c r="Y24" s="22"/>
     </row>
-    <row r="25" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B25" s="21"/>
       <c r="H25" s="22"/>
       <c r="K25" s="21"/>
@@ -4029,7 +4377,7 @@
       <c r="T25" s="21"/>
       <c r="Y25" s="22"/>
     </row>
-    <row r="26" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B26" s="21"/>
       <c r="C26" s="23" t="s">
         <v>0</v>
@@ -4045,7 +4393,7 @@
       </c>
       <c r="Y26" s="22"/>
     </row>
-    <row r="27" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B27" s="21"/>
       <c r="H27" s="22"/>
       <c r="K27" s="21"/>
@@ -4053,7 +4401,7 @@
       <c r="T27" s="21"/>
       <c r="Y27" s="22"/>
     </row>
-    <row r="28" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B28" s="21"/>
       <c r="H28" s="22"/>
       <c r="K28" s="21"/>
@@ -4061,7 +4409,7 @@
       <c r="T28" s="21"/>
       <c r="Y28" s="22"/>
     </row>
-    <row r="29" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B29" s="21"/>
       <c r="H29" s="22"/>
       <c r="K29" s="21"/>
@@ -4069,7 +4417,7 @@
       <c r="T29" s="21"/>
       <c r="Y29" s="22"/>
     </row>
-    <row r="30" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B30" s="21"/>
       <c r="H30" s="22"/>
       <c r="K30" s="21"/>
@@ -4077,7 +4425,7 @@
       <c r="T30" s="21"/>
       <c r="Y30" s="22"/>
     </row>
-    <row r="31" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B31" s="21"/>
       <c r="H31" s="22"/>
       <c r="K31" s="21"/>
@@ -4085,7 +4433,7 @@
       <c r="T31" s="21"/>
       <c r="Y31" s="22"/>
     </row>
-    <row r="32" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B32" s="21"/>
       <c r="H32" s="22"/>
       <c r="K32" s="21"/>
@@ -4093,7 +4441,7 @@
       <c r="T32" s="21"/>
       <c r="Y32" s="22"/>
     </row>
-    <row r="33" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B33" s="21"/>
       <c r="H33" s="22"/>
       <c r="K33" s="21"/>
@@ -4101,7 +4449,7 @@
       <c r="T33" s="21"/>
       <c r="Y33" s="22"/>
     </row>
-    <row r="34" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B34" s="21"/>
       <c r="H34" s="22"/>
       <c r="K34" s="21"/>
@@ -4109,7 +4457,7 @@
       <c r="T34" s="21"/>
       <c r="Y34" s="22"/>
     </row>
-    <row r="35" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B35" s="21"/>
       <c r="H35" s="22"/>
       <c r="K35" s="21"/>
@@ -4117,7 +4465,7 @@
       <c r="T35" s="21"/>
       <c r="Y35" s="22"/>
     </row>
-    <row r="36" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B36" s="21"/>
       <c r="H36" s="22"/>
       <c r="K36" s="21"/>
@@ -4125,7 +4473,7 @@
       <c r="T36" s="21"/>
       <c r="Y36" s="22"/>
     </row>
-    <row r="37" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B37" s="21"/>
       <c r="H37" s="22"/>
       <c r="K37" s="21"/>
@@ -4133,7 +4481,7 @@
       <c r="T37" s="21"/>
       <c r="Y37" s="22"/>
     </row>
-    <row r="38" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B38" s="21"/>
       <c r="H38" s="22"/>
       <c r="K38" s="21"/>
@@ -4141,7 +4489,7 @@
       <c r="T38" s="21"/>
       <c r="Y38" s="22"/>
     </row>
-    <row r="39" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B39" s="21"/>
       <c r="H39" s="22"/>
       <c r="K39" s="21"/>
@@ -4149,7 +4497,7 @@
       <c r="T39" s="21"/>
       <c r="Y39" s="22"/>
     </row>
-    <row r="40" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B40" s="21"/>
       <c r="H40" s="22"/>
       <c r="K40" s="21"/>
@@ -4157,7 +4505,7 @@
       <c r="T40" s="21"/>
       <c r="Y40" s="22"/>
     </row>
-    <row r="41" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B41" s="21"/>
       <c r="H41" s="22"/>
       <c r="K41" s="21"/>
@@ -4165,7 +4513,7 @@
       <c r="T41" s="21"/>
       <c r="Y41" s="22"/>
     </row>
-    <row r="42" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B42" s="21"/>
       <c r="H42" s="22"/>
       <c r="K42" s="21"/>
@@ -4173,7 +4521,7 @@
       <c r="T42" s="21"/>
       <c r="Y42" s="22"/>
     </row>
-    <row r="43" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B43" s="21"/>
       <c r="H43" s="22"/>
       <c r="K43" s="21"/>
@@ -4181,7 +4529,7 @@
       <c r="T43" s="21"/>
       <c r="Y43" s="22"/>
     </row>
-    <row r="44" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B44" s="21"/>
       <c r="C44" s="23" t="s">
         <v>16</v>
@@ -4197,7 +4545,7 @@
       </c>
       <c r="Y44" s="22"/>
     </row>
-    <row r="45" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B45" s="21"/>
       <c r="H45" s="22"/>
       <c r="K45" s="21"/>
@@ -4205,7 +4553,7 @@
       <c r="T45" s="21"/>
       <c r="Y45" s="22"/>
     </row>
-    <row r="46" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B46" s="21"/>
       <c r="H46" s="22"/>
       <c r="K46" s="21"/>
@@ -4213,7 +4561,7 @@
       <c r="T46" s="21"/>
       <c r="Y46" s="22"/>
     </row>
-    <row r="47" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B47" s="21"/>
       <c r="H47" s="22"/>
       <c r="K47" s="21"/>
@@ -4221,7 +4569,7 @@
       <c r="T47" s="21"/>
       <c r="Y47" s="22"/>
     </row>
-    <row r="48" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B48" s="21"/>
       <c r="H48" s="22"/>
       <c r="K48" s="21"/>
@@ -4229,7 +4577,7 @@
       <c r="T48" s="21"/>
       <c r="Y48" s="22"/>
     </row>
-    <row r="49" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B49" s="21"/>
       <c r="H49" s="22"/>
       <c r="K49" s="21"/>
@@ -4237,7 +4585,7 @@
       <c r="T49" s="21"/>
       <c r="Y49" s="22"/>
     </row>
-    <row r="50" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B50" s="21"/>
       <c r="H50" s="22"/>
       <c r="K50" s="21"/>
@@ -4245,7 +4593,7 @@
       <c r="T50" s="21"/>
       <c r="Y50" s="22"/>
     </row>
-    <row r="51" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B51" s="21"/>
       <c r="H51" s="22"/>
       <c r="K51" s="21"/>
@@ -4253,7 +4601,7 @@
       <c r="T51" s="21"/>
       <c r="Y51" s="22"/>
     </row>
-    <row r="52" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B52" s="21"/>
       <c r="H52" s="22"/>
       <c r="K52" s="21"/>
@@ -4261,7 +4609,7 @@
       <c r="T52" s="21"/>
       <c r="Y52" s="22"/>
     </row>
-    <row r="53" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B53" s="21"/>
       <c r="H53" s="22"/>
       <c r="K53" s="21"/>
@@ -4269,7 +4617,7 @@
       <c r="T53" s="21"/>
       <c r="Y53" s="22"/>
     </row>
-    <row r="54" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B54" s="21"/>
       <c r="H54" s="22"/>
       <c r="K54" s="21"/>
@@ -4277,7 +4625,7 @@
       <c r="T54" s="21"/>
       <c r="Y54" s="22"/>
     </row>
-    <row r="55" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B55" s="21"/>
       <c r="H55" s="22"/>
       <c r="K55" s="21"/>
@@ -4285,7 +4633,7 @@
       <c r="T55" s="21"/>
       <c r="Y55" s="22"/>
     </row>
-    <row r="56" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B56" s="21"/>
       <c r="H56" s="22"/>
       <c r="K56" s="21"/>
@@ -4293,7 +4641,7 @@
       <c r="T56" s="21"/>
       <c r="Y56" s="22"/>
     </row>
-    <row r="57" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B57" s="21"/>
       <c r="H57" s="22"/>
       <c r="K57" s="21"/>
@@ -4301,7 +4649,7 @@
       <c r="T57" s="21"/>
       <c r="Y57" s="22"/>
     </row>
-    <row r="58" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B58" s="21"/>
       <c r="H58" s="22"/>
       <c r="K58" s="21"/>
@@ -4309,7 +4657,7 @@
       <c r="T58" s="21"/>
       <c r="Y58" s="22"/>
     </row>
-    <row r="59" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B59" s="21"/>
       <c r="H59" s="22"/>
       <c r="K59" s="21"/>
@@ -4317,7 +4665,7 @@
       <c r="T59" s="21"/>
       <c r="Y59" s="22"/>
     </row>
-    <row r="60" spans="2:25" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B60" s="21"/>
       <c r="H60" s="22"/>
       <c r="K60" s="21"/>
@@ -4325,7 +4673,7 @@
       <c r="T60" s="21"/>
       <c r="Y60" s="22"/>
     </row>
-    <row r="61" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B61" s="24"/>
       <c r="C61" s="25"/>
       <c r="D61" s="25"/>
@@ -4343,7 +4691,7 @@
       <c r="T61" s="21"/>
       <c r="Y61" s="22"/>
     </row>
-    <row r="62" spans="2:25" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:25" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="T62" s="24"/>
       <c r="U62" s="25"/>
       <c r="V62" s="25"/>
@@ -4371,17 +4719,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F4196E-D435-064A-B41B-979B9B2AEE8B}">
   <dimension ref="B3:J20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="17.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>8</v>
       </c>
@@ -4401,52 +4749,52 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B5" s="38">
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="16">
         <v>4</v>
       </c>
-      <c r="C5" s="37">
+      <c r="C5" s="11">
         <v>1.0810999999999999</v>
       </c>
-      <c r="D5" s="37">
+      <c r="D5" s="11">
         <v>0.75480199999999997</v>
       </c>
-      <c r="E5" s="37">
+      <c r="E5" s="11">
         <v>0.75643000000000005</v>
       </c>
-      <c r="F5" s="37">
+      <c r="F5" s="11">
         <v>0.75480199999999997</v>
       </c>
-      <c r="G5" s="39">
+      <c r="G5" s="12">
         <v>0.75505</v>
       </c>
     </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B6" s="40">
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6">
         <v>10</v>
       </c>
-      <c r="C6" s="40">
+      <c r="C6">
         <v>1.7057</v>
       </c>
-      <c r="D6" s="40">
+      <c r="D6">
         <v>0.76384099999999999</v>
       </c>
-      <c r="E6" s="40">
+      <c r="E6">
         <v>0.76824000000000003</v>
       </c>
-      <c r="F6" s="40">
+      <c r="F6">
         <v>0.76383999999999996</v>
       </c>
-      <c r="G6" s="40">
+      <c r="G6">
         <v>0.76429000000000002</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="J20" t="s">
         <v>38</v>
       </c>
@@ -4458,4 +4806,1304 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3514071E-FCF0-470F-B09E-BE50D5490F60}">
+  <dimension ref="A1:Q24"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="9" max="13" width="19.375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="23.125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I1" t="s">
+        <v>47</v>
+      </c>
+      <c r="J1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L1" t="s">
+        <v>50</v>
+      </c>
+      <c r="M1" t="s">
+        <v>51</v>
+      </c>
+      <c r="N1" t="s">
+        <v>52</v>
+      </c>
+      <c r="O1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2">
+        <v>0.1</v>
+      </c>
+      <c r="E2">
+        <v>200000</v>
+      </c>
+      <c r="F2">
+        <v>0.01</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>16</v>
+      </c>
+      <c r="I2" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="J2" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="K2" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="L2" s="37" t="s">
+        <v>61</v>
+      </c>
+      <c r="M2" s="37" t="s">
+        <v>62</v>
+      </c>
+      <c r="N2">
+        <v>5.7843999999999998</v>
+      </c>
+      <c r="O2">
+        <v>152.99700000000001</v>
+      </c>
+      <c r="P2">
+        <v>9.6809999999999992</v>
+      </c>
+      <c r="Q2" s="37" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>0.1</v>
+      </c>
+      <c r="E3">
+        <v>200000</v>
+      </c>
+      <c r="F3">
+        <v>0.3</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3" s="37" t="s">
+        <v>64</v>
+      </c>
+      <c r="J3" s="37" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="L3">
+        <v>0.74350282485875696</v>
+      </c>
+      <c r="M3" s="37" t="s">
+        <v>67</v>
+      </c>
+      <c r="N3">
+        <v>5.7117000000000004</v>
+      </c>
+      <c r="O3">
+        <v>154.946</v>
+      </c>
+      <c r="P3">
+        <v>19.434000000000001</v>
+      </c>
+      <c r="Q3" s="37" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>0.3</v>
+      </c>
+      <c r="E4">
+        <v>200000</v>
+      </c>
+      <c r="F4">
+        <v>0.01</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>32</v>
+      </c>
+      <c r="I4">
+        <v>0.832081139087677</v>
+      </c>
+      <c r="J4">
+        <v>0.71186440677966101</v>
+      </c>
+      <c r="K4" s="37" t="s">
+        <v>69</v>
+      </c>
+      <c r="L4" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="M4" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="N4">
+        <v>5.6421999999999999</v>
+      </c>
+      <c r="O4">
+        <v>156.85300000000001</v>
+      </c>
+      <c r="P4">
+        <v>4.9630000000000001</v>
+      </c>
+      <c r="Q4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5">
+        <v>10</v>
+      </c>
+      <c r="D5">
+        <v>0.3</v>
+      </c>
+      <c r="E5">
+        <v>200000</v>
+      </c>
+      <c r="F5">
+        <v>0.01</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>8</v>
+      </c>
+      <c r="I5" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="J5">
+        <v>0.75141242937853103</v>
+      </c>
+      <c r="K5" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="L5">
+        <v>0.75141242937853103</v>
+      </c>
+      <c r="M5" s="37" t="s">
+        <v>74</v>
+      </c>
+      <c r="N5">
+        <v>5.7222</v>
+      </c>
+      <c r="O5">
+        <v>154.66</v>
+      </c>
+      <c r="P5">
+        <v>19.398</v>
+      </c>
+      <c r="Q5" s="37" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6">
+        <v>10</v>
+      </c>
+      <c r="D6">
+        <v>0.5</v>
+      </c>
+      <c r="E6">
+        <v>200000</v>
+      </c>
+      <c r="F6">
+        <v>0.01</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>8</v>
+      </c>
+      <c r="I6" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="J6" s="37" t="s">
+        <v>76</v>
+      </c>
+      <c r="K6" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="L6" s="37" t="s">
+        <v>78</v>
+      </c>
+      <c r="M6" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="N6">
+        <v>5.7435</v>
+      </c>
+      <c r="O6">
+        <v>154.08799999999999</v>
+      </c>
+      <c r="P6">
+        <v>19.326000000000001</v>
+      </c>
+      <c r="Q6" s="37" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>0.1</v>
+      </c>
+      <c r="E7">
+        <v>200000</v>
+      </c>
+      <c r="F7">
+        <v>0.01</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>16</v>
+      </c>
+      <c r="I7" s="37" t="s">
+        <v>80</v>
+      </c>
+      <c r="J7" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="K7" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="L7" s="37" t="s">
+        <v>83</v>
+      </c>
+      <c r="M7">
+        <v>0.70337717108389097</v>
+      </c>
+      <c r="N7">
+        <v>5.8090000000000002</v>
+      </c>
+      <c r="O7">
+        <v>152.34899999999999</v>
+      </c>
+      <c r="P7">
+        <v>9.64</v>
+      </c>
+      <c r="Q7" s="37" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8">
+        <v>0.1</v>
+      </c>
+      <c r="E8">
+        <v>200000</v>
+      </c>
+      <c r="F8">
+        <v>0.01</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>8</v>
+      </c>
+      <c r="I8" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="J8" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="K8">
+        <v>0.73896113723615897</v>
+      </c>
+      <c r="L8" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="M8" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="N8">
+        <v>5.0194000000000001</v>
+      </c>
+      <c r="O8">
+        <v>176.316</v>
+      </c>
+      <c r="P8">
+        <v>22.114000000000001</v>
+      </c>
+      <c r="Q8" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9">
+        <v>5</v>
+      </c>
+      <c r="D9">
+        <v>0.1</v>
+      </c>
+      <c r="E9">
+        <v>200000</v>
+      </c>
+      <c r="F9">
+        <v>0.3</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>8</v>
+      </c>
+      <c r="I9" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="J9" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="K9" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="L9" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="M9" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="N9">
+        <v>5.7933000000000003</v>
+      </c>
+      <c r="O9">
+        <v>152.762</v>
+      </c>
+      <c r="P9">
+        <v>19.16</v>
+      </c>
+      <c r="Q9" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10">
+        <v>5</v>
+      </c>
+      <c r="D10">
+        <v>0.3</v>
+      </c>
+      <c r="E10">
+        <v>200000</v>
+      </c>
+      <c r="F10">
+        <v>0.01</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>32</v>
+      </c>
+      <c r="I10">
+        <v>0.829886794090271</v>
+      </c>
+      <c r="J10" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="K10" s="37" t="s">
+        <v>96</v>
+      </c>
+      <c r="L10" s="37" t="s">
+        <v>95</v>
+      </c>
+      <c r="M10" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="N10">
+        <v>53.015799999999999</v>
+      </c>
+      <c r="O10">
+        <v>16.693000000000001</v>
+      </c>
+      <c r="P10">
+        <v>0.52800000000000002</v>
+      </c>
+      <c r="Q10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11">
+        <v>0.3</v>
+      </c>
+      <c r="E11">
+        <v>200000</v>
+      </c>
+      <c r="F11">
+        <v>0.01</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>8</v>
+      </c>
+      <c r="I11" s="37" t="s">
+        <v>98</v>
+      </c>
+      <c r="J11" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="K11">
+        <v>0.73855942930280605</v>
+      </c>
+      <c r="L11" s="37" t="s">
+        <v>99</v>
+      </c>
+      <c r="M11">
+        <v>0.73366349556050003</v>
+      </c>
+      <c r="N11">
+        <v>5.7241</v>
+      </c>
+      <c r="O11">
+        <v>154.608</v>
+      </c>
+      <c r="P11">
+        <v>19.391999999999999</v>
+      </c>
+      <c r="Q11" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12">
+        <v>5</v>
+      </c>
+      <c r="D12">
+        <v>0.5</v>
+      </c>
+      <c r="E12">
+        <v>200000</v>
+      </c>
+      <c r="F12">
+        <v>0.01</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>8</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="J12">
+        <v>0.735593220338983</v>
+      </c>
+      <c r="K12" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="L12">
+        <v>0.735593220338983</v>
+      </c>
+      <c r="M12" s="37" t="s">
+        <v>102</v>
+      </c>
+      <c r="N12">
+        <v>5.7842000000000002</v>
+      </c>
+      <c r="O12">
+        <v>153.00200000000001</v>
+      </c>
+      <c r="P12">
+        <v>19.190000000000001</v>
+      </c>
+      <c r="Q12" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C13">
+        <v>10</v>
+      </c>
+      <c r="D13">
+        <v>0.1</v>
+      </c>
+      <c r="E13">
+        <v>200000</v>
+      </c>
+      <c r="F13">
+        <v>0.01</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>16</v>
+      </c>
+      <c r="I13" s="37" t="s">
+        <v>104</v>
+      </c>
+      <c r="J13" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="K13" s="37" t="s">
+        <v>106</v>
+      </c>
+      <c r="L13" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="M13" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="N13">
+        <v>12.3764</v>
+      </c>
+      <c r="O13">
+        <v>71.507000000000005</v>
+      </c>
+      <c r="P13">
+        <v>4.5250000000000004</v>
+      </c>
+      <c r="Q13" s="37" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" t="s">
+        <v>103</v>
+      </c>
+      <c r="C14">
+        <v>10</v>
+      </c>
+      <c r="D14">
+        <v>0.1</v>
+      </c>
+      <c r="E14">
+        <v>200000</v>
+      </c>
+      <c r="F14">
+        <v>0.01</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>8</v>
+      </c>
+      <c r="I14" s="37" t="s">
+        <v>108</v>
+      </c>
+      <c r="J14" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="K14" s="37" t="s">
+        <v>110</v>
+      </c>
+      <c r="L14" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="M14" s="37" t="s">
+        <v>111</v>
+      </c>
+      <c r="N14">
+        <v>10.6198</v>
+      </c>
+      <c r="O14">
+        <v>83.334999999999994</v>
+      </c>
+      <c r="P14">
+        <v>10.452</v>
+      </c>
+      <c r="Q14" s="37" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C15">
+        <v>10</v>
+      </c>
+      <c r="D15">
+        <v>0.1</v>
+      </c>
+      <c r="E15">
+        <v>200000</v>
+      </c>
+      <c r="F15">
+        <v>0.3</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>8</v>
+      </c>
+      <c r="I15" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="J15">
+        <v>0.8</v>
+      </c>
+      <c r="K15">
+        <v>0.80396146624901799</v>
+      </c>
+      <c r="L15">
+        <v>0.8</v>
+      </c>
+      <c r="M15" s="37" t="s">
+        <v>113</v>
+      </c>
+      <c r="N15">
+        <v>10.8192</v>
+      </c>
+      <c r="O15">
+        <v>81.799000000000007</v>
+      </c>
+      <c r="P15">
+        <v>10.26</v>
+      </c>
+      <c r="Q15" s="37" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16">
+        <v>10</v>
+      </c>
+      <c r="D16">
+        <v>0.3</v>
+      </c>
+      <c r="E16">
+        <v>200000</v>
+      </c>
+      <c r="F16">
+        <v>0.01</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>32</v>
+      </c>
+      <c r="I16" s="37" t="s">
+        <v>114</v>
+      </c>
+      <c r="J16" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="K16" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="L16" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="M16" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="N16">
+        <v>10.6526</v>
+      </c>
+      <c r="O16">
+        <v>83.078000000000003</v>
+      </c>
+      <c r="P16">
+        <v>2.6280000000000001</v>
+      </c>
+      <c r="Q16">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" t="s">
+        <v>103</v>
+      </c>
+      <c r="C17">
+        <v>10</v>
+      </c>
+      <c r="D17">
+        <v>0.3</v>
+      </c>
+      <c r="E17">
+        <v>200000</v>
+      </c>
+      <c r="F17">
+        <v>0.01</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>8</v>
+      </c>
+      <c r="I17" s="37" t="s">
+        <v>119</v>
+      </c>
+      <c r="J17" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="K17" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="L17" s="37" t="s">
+        <v>121</v>
+      </c>
+      <c r="M17" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="N17">
+        <v>9.9415999999999993</v>
+      </c>
+      <c r="O17">
+        <v>89.019000000000005</v>
+      </c>
+      <c r="P17">
+        <v>11.164999999999999</v>
+      </c>
+      <c r="Q17" s="37" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18">
+        <v>10</v>
+      </c>
+      <c r="D18">
+        <v>0.5</v>
+      </c>
+      <c r="E18">
+        <v>200000</v>
+      </c>
+      <c r="F18">
+        <v>0.01</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>8</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>123</v>
+      </c>
+      <c r="J18" s="37" t="s">
+        <v>124</v>
+      </c>
+      <c r="K18" s="37" t="s">
+        <v>125</v>
+      </c>
+      <c r="L18" s="37" t="s">
+        <v>124</v>
+      </c>
+      <c r="M18" s="37" t="s">
+        <v>126</v>
+      </c>
+      <c r="N18">
+        <v>9.9001000000000001</v>
+      </c>
+      <c r="O18">
+        <v>89.393000000000001</v>
+      </c>
+      <c r="P18">
+        <v>11.212</v>
+      </c>
+      <c r="Q18" s="37" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19">
+        <v>5</v>
+      </c>
+      <c r="D19">
+        <v>0.1</v>
+      </c>
+      <c r="E19">
+        <v>200000</v>
+      </c>
+      <c r="F19">
+        <v>0.01</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>16</v>
+      </c>
+      <c r="I19" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="J19" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="K19" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="L19" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="M19" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="N19">
+        <v>9.9293999999999993</v>
+      </c>
+      <c r="O19">
+        <v>89.129000000000005</v>
+      </c>
+      <c r="P19">
+        <v>5.64</v>
+      </c>
+      <c r="Q19" s="37" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20">
+        <v>5</v>
+      </c>
+      <c r="D20">
+        <v>0.1</v>
+      </c>
+      <c r="E20">
+        <v>200000</v>
+      </c>
+      <c r="F20">
+        <v>0.01</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>8</v>
+      </c>
+      <c r="I20" s="37" t="s">
+        <v>131</v>
+      </c>
+      <c r="J20" s="37" t="s">
+        <v>132</v>
+      </c>
+      <c r="K20">
+        <v>0.78744903449612502</v>
+      </c>
+      <c r="L20" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="M20" s="37" t="s">
+        <v>134</v>
+      </c>
+      <c r="N20">
+        <v>9.8615999999999993</v>
+      </c>
+      <c r="O20">
+        <v>89.742000000000004</v>
+      </c>
+      <c r="P20">
+        <v>11.256</v>
+      </c>
+      <c r="Q20" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21" t="s">
+        <v>103</v>
+      </c>
+      <c r="C21">
+        <v>5</v>
+      </c>
+      <c r="D21">
+        <v>0.1</v>
+      </c>
+      <c r="E21">
+        <v>200000</v>
+      </c>
+      <c r="F21">
+        <v>0.3</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>8</v>
+      </c>
+      <c r="I21" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="J21" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="K21" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="L21" s="37" t="s">
+        <v>138</v>
+      </c>
+      <c r="M21" s="37" t="s">
+        <v>139</v>
+      </c>
+      <c r="N21">
+        <v>9.7594999999999992</v>
+      </c>
+      <c r="O21">
+        <v>90.680999999999997</v>
+      </c>
+      <c r="P21">
+        <v>11.372999999999999</v>
+      </c>
+      <c r="Q21" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" t="s">
+        <v>103</v>
+      </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+      <c r="D22">
+        <v>0.3</v>
+      </c>
+      <c r="E22">
+        <v>200000</v>
+      </c>
+      <c r="F22">
+        <v>0.01</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22">
+        <v>32</v>
+      </c>
+      <c r="I22" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="J22" s="37" t="s">
+        <v>141</v>
+      </c>
+      <c r="K22">
+        <v>0.77448623990574506</v>
+      </c>
+      <c r="L22" s="37" t="s">
+        <v>141</v>
+      </c>
+      <c r="M22" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="N22">
+        <v>60.653399999999998</v>
+      </c>
+      <c r="O22">
+        <v>14.590999999999999</v>
+      </c>
+      <c r="P22">
+        <v>0.46200000000000002</v>
+      </c>
+      <c r="Q22">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" t="s">
+        <v>103</v>
+      </c>
+      <c r="C23">
+        <v>5</v>
+      </c>
+      <c r="D23">
+        <v>0.3</v>
+      </c>
+      <c r="E23">
+        <v>200000</v>
+      </c>
+      <c r="F23">
+        <v>0.01</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>8</v>
+      </c>
+      <c r="I23" s="37" t="s">
+        <v>143</v>
+      </c>
+      <c r="J23" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="K23" s="37" t="s">
+        <v>144</v>
+      </c>
+      <c r="L23" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="M23" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="N23">
+        <v>9.8535000000000004</v>
+      </c>
+      <c r="O23">
+        <v>89.816000000000003</v>
+      </c>
+      <c r="P23">
+        <v>11.265000000000001</v>
+      </c>
+      <c r="Q23" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24" t="s">
+        <v>103</v>
+      </c>
+      <c r="C24">
+        <v>5</v>
+      </c>
+      <c r="D24">
+        <v>0.5</v>
+      </c>
+      <c r="E24">
+        <v>200000</v>
+      </c>
+      <c r="F24">
+        <v>0.01</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24">
+        <v>8</v>
+      </c>
+      <c r="I24" s="37" t="s">
+        <v>146</v>
+      </c>
+      <c r="J24" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="K24" s="37" t="s">
+        <v>144</v>
+      </c>
+      <c r="L24" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="M24" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="N24">
+        <v>9.8381000000000007</v>
+      </c>
+      <c r="O24">
+        <v>89.956000000000003</v>
+      </c>
+      <c r="P24">
+        <v>11.282999999999999</v>
+      </c>
+      <c r="Q24" s="37" t="s">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update experimenets excels
</commit_message>
<xml_diff>
--- a/ExperimentsData.xlsx
+++ b/ExperimentsData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GithubProjects\prethesis-experiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04519A7D-8A07-4F8A-93CA-075913036BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38FC04D-553E-44FA-9423-16F222CD58B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="6" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="6" xr2:uid="{D2947EBA-2734-2E4C-9794-385CE60DBACE}"/>
   </bookViews>
   <sheets>
     <sheet name="Dataset Distribution" sheetId="4" r:id="rId1"/>
@@ -320,7 +320,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="229">
   <si>
     <t>DistilBERT</t>
   </si>
@@ -992,6 +992,21 @@
   </si>
   <si>
     <t>1.178574562072754</t>
+  </si>
+  <si>
+    <t>BAGGING</t>
+  </si>
+  <si>
+    <t>Combination</t>
+  </si>
+  <si>
+    <t>IndoBERT + DistilBERT</t>
+  </si>
+  <si>
+    <t>F1-Score</t>
+  </si>
+  <si>
+    <t>Two IndoBERT</t>
   </si>
 </sst>
 </file>
@@ -1294,7 +1309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1361,6 +1376,25 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -6374,12 +6408,12 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50CEE2EF-92BC-4D8D-9328-6DE9B89DE831}">
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="59.75" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" customWidth="1"/>
     <col min="4" max="4" width="9.125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.875" bestFit="1" customWidth="1"/>
@@ -7665,7 +7699,53 @@
         <v>150</v>
       </c>
     </row>
+    <row r="27" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C27" s="23" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C28" s="38" t="s">
+        <v>225</v>
+      </c>
+      <c r="D28" s="39"/>
+      <c r="E28" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F28" s="20" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C29" s="40" t="s">
+        <v>226</v>
+      </c>
+      <c r="D29" s="41"/>
+      <c r="E29" s="42">
+        <v>0.77180000000000004</v>
+      </c>
+      <c r="F29" s="22">
+        <v>0.7722</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C30" s="43" t="s">
+        <v>228</v>
+      </c>
+      <c r="D30" s="44"/>
+      <c r="E30" s="25">
+        <v>0.77290000000000003</v>
+      </c>
+      <c r="F30" s="26">
+        <v>0.77370000000000005</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C30:D30"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>